<commit_message>
add employee_id for excel
</commit_message>
<xml_diff>
--- a/xlsx/asset_import_template (2).xlsx
+++ b/xlsx/asset_import_template (2).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t xml:space="preserve">Название</t>
   </si>
@@ -52,12 +52,6 @@
     <t xml:space="preserve">Период проверки</t>
   </si>
   <si>
-    <t xml:space="preserve">Табельный номер</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ФИО</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ботинки без м/ч 42 </t>
   </si>
   <si>
@@ -74,9 +68,6 @@
   </si>
   <si>
     <t xml:space="preserve">2024-10-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Малых Андрей</t>
   </si>
 </sst>
 </file>
@@ -360,7 +351,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.39"/>
@@ -408,46 +399,34 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="I2" s="1" t="n">
         <v>365</v>
       </c>
       <c r="J2" s="1" t="n">
         <v>30</v>
-      </c>
-      <c r="K2" s="1" t="n">
-        <v>10680</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add export for inventory
</commit_message>
<xml_diff>
--- a/xlsx/asset_import_template (2).xlsx
+++ b/xlsx/asset_import_template (2).xlsx
@@ -20,58 +20,69 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t xml:space="preserve">Название</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Инвентарный номер</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Серийный номер</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t xml:space="preserve">Инвентарный номер / Inventory number</t>
   </si>
   <si>
     <t xml:space="preserve">Комментарий</t>
   </si>
   <si>
-    <t xml:space="preserve">Дата выпуска</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дата покупки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дата обслуживания</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Период обслуживания</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Период проверки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПК</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Выдан сотруднику отдела разработки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-10-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-09-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-10-01</t>
+    <t xml:space="preserve">Тип и модель ПК / PC type and model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Серийный номер / Serial Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата выдачи / Issue Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата покупки / Purchasing Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата обслуживания / Service date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Период обслуживания / 
+Service period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Период проверки / Check period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop,mouse,bag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lenovo ThinkBook 15 G4 IAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MP2KDZYH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 18.12.2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop,mouse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop Acer Extensa 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NXEGYER00H32008A5D3400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 27.03.2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -98,6 +109,27 @@
       <charset val="204"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF413003"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="12"/>
       <color theme="1"/>
@@ -105,16 +137,53 @@
       <family val="1"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFBF0"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FF993300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0E0E3"/>
+        <bgColor rgb="FFCCFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFF99"/>
+        <bgColor rgb="FFFFFF99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FFC0C0C0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -122,6 +191,13 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -148,7 +224,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -157,12 +233,48 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -174,7 +286,172 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFBF0"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFD0E0E3"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFF99"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF92D050"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF413003"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>798480</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>236160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>644760</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>60120</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1" name="Text Box 4" hidden="1"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="798480" y="927000"/>
+          <a:ext cx="9839880" cy="2990160"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFE1"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:miter/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw algn="ctr" dir="2700000" dist="35638" rotWithShape="0">
+            <a:srgbClr val="000000"/>
+          </a:outerShdw>
+        </a:effectLst>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>798480</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>236160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>644760</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>60120</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Text Box 1" hidden="1"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="798480" y="927000"/>
+          <a:ext cx="9839880" cy="2228040"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFE1"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:miter/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw algn="ctr" dir="2700000" dist="35638" rotWithShape="0">
+            <a:srgbClr val="000000"/>
+          </a:outerShdw>
+        </a:effectLst>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -357,7 +634,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.39"/>
@@ -371,64 +648,243 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="17.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="17.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="14.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="54.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="41.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="n">
+        <v>100000002700</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>140000191</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="C2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="D2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="E2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="F2" s="10"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+    </row>
+    <row r="3" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="n">
+        <v>100000003372</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="1" t="n">
-        <v>365</v>
-      </c>
-      <c r="I2" s="1" t="n">
-        <v>30</v>
-      </c>
+      <c r="C3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="12" t="n">
+        <v>2024</v>
+      </c>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
     </row>
+    <row r="1048416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048418" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048419" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048420" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048421" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048422" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048423" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048424" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048425" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048426" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048427" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048428" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048429" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048430" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048431" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048432" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048433" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048434" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048435" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048436" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048437" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048438" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048439" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048440" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048441" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048442" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048443" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048444" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048445" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048446" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048447" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048448" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048449" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048450" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048451" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048452" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048453" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048454" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048455" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048456" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048457" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048458" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048459" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048460" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048461" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048462" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048463" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048464" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048465" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048466" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048467" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048468" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048469" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048470" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048471" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048472" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048473" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048474" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048475" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048476" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048477" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048478" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048479" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048480" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048481" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048482" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048483" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048484" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048485" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048486" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048487" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048488" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048489" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048490" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048491" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048492" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048493" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048494" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048495" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048496" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048497" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048498" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048499" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048500" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048501" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048502" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048503" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048504" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048505" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048506" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048507" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048508" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048509" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048510" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048511" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048512" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048513" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048514" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048515" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048516" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048517" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048518" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048519" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048520" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048521" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048522" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048523" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048524" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048525" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048526" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048527" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048528" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048529" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048530" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048531" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048532" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048533" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048534" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048535" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048536" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048537" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048538" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048539" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048540" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048541" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048542" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048543" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -437,5 +893,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
edit save asset location
</commit_message>
<xml_diff>
--- a/xlsx/asset_import_template (2).xlsx
+++ b/xlsx/asset_import_template (2).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">Инвентарный номер / Inventory number</t>
   </si>
@@ -72,6 +72,12 @@
   </si>
   <si>
     <t xml:space="preserve">Акт 27.03.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ноутбук 15.6\" MSI Modern 15 F13MG </t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2410N0009256 </t>
   </si>
 </sst>
 </file>
@@ -224,7 +230,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -275,6 +281,10 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -356,13 +366,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>798480</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>236160</xdr:rowOff>
+      <xdr:rowOff>424800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>644760</xdr:colOff>
+      <xdr:colOff>644400</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>60120</xdr:rowOff>
+      <xdr:rowOff>30600</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -372,7 +382,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="798480" y="927000"/>
-          <a:ext cx="9839880" cy="2990160"/>
+          <a:ext cx="9839520" cy="2989800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -406,13 +416,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>798480</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>236160</xdr:rowOff>
+      <xdr:rowOff>424800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>644760</xdr:colOff>
+      <xdr:colOff>644400</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>60120</xdr:rowOff>
+      <xdr:rowOff>30600</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -422,7 +432,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="798480" y="927000"/>
-          <a:ext cx="9839880" cy="2228040"/>
+          <a:ext cx="9839520" cy="2227680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -651,7 +661,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="54.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -680,7 +690,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="41.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="n">
         <v>100000002700</v>
       </c>
@@ -701,7 +711,7 @@
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
     </row>
-    <row r="3" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="n">
         <v>100000003372</v>
       </c>
@@ -723,6 +733,17 @@
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
+    </row>
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="n">
+        <v>100000004480</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="1048416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
add AI for excel import
</commit_message>
<xml_diff>
--- a/xlsx/asset_import_template (2).xlsx
+++ b/xlsx/asset_import_template (2).xlsx
@@ -77,7 +77,7 @@
     <t xml:space="preserve">Ноутбук 15.6\" MSI Modern 15 F13MG </t>
   </si>
   <si>
-    <t xml:space="preserve">C2410N0009256 </t>
+    <t xml:space="preserve">C2410N0009256</t>
   </si>
 </sst>
 </file>
@@ -283,7 +283,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -370,9 +370,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>644400</xdr:colOff>
+      <xdr:colOff>644040</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>30600</xdr:rowOff>
+      <xdr:rowOff>30240</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -382,7 +382,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="798480" y="927000"/>
-          <a:ext cx="9839520" cy="2989800"/>
+          <a:ext cx="9839160" cy="2989440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -420,9 +420,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>644400</xdr:colOff>
+      <xdr:colOff>644040</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>30600</xdr:rowOff>
+      <xdr:rowOff>30240</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -432,7 +432,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="798480" y="927000"/>
-          <a:ext cx="9839520" cy="2227680"/>
+          <a:ext cx="9839160" cy="2227320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -736,7 +736,7 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="n">
-        <v>100000004480</v>
+        <v>10000000448011</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
protection inv_id and sn by from null
</commit_message>
<xml_diff>
--- a/xlsx/asset_import_template (2).xlsx
+++ b/xlsx/asset_import_template (2).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t xml:space="preserve">Инвентарный номер / Inventory number</t>
   </si>
@@ -50,48 +50,22 @@
     <t xml:space="preserve">Период проверки / Check period</t>
   </si>
   <si>
-    <t xml:space="preserve">Laptop,mouse,bag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lenovo ThinkBook 15 G4 IAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MP2KDZYH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Акт 18.12.2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laptop,mouse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laptop Acer Extensa 15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NXEGYER00H32008A5D3400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Акт 27.03.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Создаем с нуля</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ноутбук 15.6\" MSI Modern 15 F13MG </t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2410N0009256</t>
+    <t xml:space="preserve">GGGG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вапифащгп ш</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -138,23 +112,8 @@
       <family val="1"/>
       <charset val="1"/>
     </font>
-    <font>
-      <b val="true"/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -171,24 +130,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
         <bgColor rgb="FF993300"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD0E0E3"/>
-        <bgColor rgb="FFCCFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCCFF99"/>
-        <bgColor rgb="FFFFFF99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor rgb="FFC0C0C0"/>
       </patternFill>
     </fill>
   </fills>
@@ -233,7 +174,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -262,32 +203,8 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -324,7 +241,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFD0E0E3"/>
+      <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -335,7 +252,7 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFF99"/>
+      <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -343,7 +260,7 @@
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF92D050"/>
+      <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -368,14 +285,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>798480</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>424800</xdr:rowOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>43560</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>644040</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>30240</xdr:rowOff>
+      <xdr:colOff>386640</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>175320</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -385,7 +302,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="798480" y="927000"/>
-          <a:ext cx="9839160" cy="2989440"/>
+          <a:ext cx="9838800" cy="2989080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -418,14 +335,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>798480</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>424800</xdr:rowOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>43560</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>644040</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>30240</xdr:rowOff>
+      <xdr:colOff>386640</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>175320</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -435,7 +352,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="798480" y="927000"/>
-          <a:ext cx="9839160" cy="2227320"/>
+          <a:ext cx="9838800" cy="2226960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -651,7 +568,7 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.4"/>
@@ -693,64 +610,112 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
-        <v>100000002700</v>
-      </c>
-      <c r="B2" s="8" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="10"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
+      <c r="E2" s="7" t="n">
+        <v>57483</v>
+      </c>
     </row>
-    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
-        <v>100000003372</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="12" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-    </row>
-    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="n">
-        <v>10000000448011</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>19</v>
-      </c>
-    </row>
+    <row r="1048321" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048322" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048323" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048324" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048325" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048326" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048327" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048328" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048329" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048330" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048331" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048332" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048333" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048334" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048335" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048336" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048337" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048338" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048339" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048340" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048341" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048342" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048343" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048344" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048345" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048346" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048347" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048348" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048349" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048350" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048352" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048353" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048354" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048356" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048357" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048358" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048359" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048360" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048361" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048362" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048363" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048364" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048365" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048366" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048367" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048368" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048369" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048370" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048371" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048372" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048373" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048374" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048375" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048376" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048377" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048379" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048380" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048381" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048382" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048383" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048384" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048385" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048386" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048387" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048389" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048390" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048391" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048392" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048394" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048395" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048396" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048397" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048398" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048399" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048400" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048401" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048402" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048403" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048404" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048405" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048406" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048407" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048408" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048409" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048410" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048411" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048412" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048413" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048414" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048415" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048418" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
edit AssetBase for AssetCreate
</commit_message>
<xml_diff>
--- a/xlsx/asset_import_template (2).xlsx
+++ b/xlsx/asset_import_template (2).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="49">
   <si>
     <t xml:space="preserve">Инвентарный номер / Inventory number</t>
   </si>
@@ -50,22 +50,139 @@
     <t xml:space="preserve">Период проверки / Check period</t>
   </si>
   <si>
-    <t xml:space="preserve">GGGG</t>
+    <t xml:space="preserve">140000257</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WorkStation,mouse,keyboard, monitor Lenovo 2424d ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workstation Lenovo ThinkStation P 320</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC10AS96</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 28.11.2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">140000420</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WorkStation,monitor(Lenovo T2324dC),mouse,keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рабочая станция Lenovo ThinkStation P310+монитор</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S4BP0263</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 14.08.2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150000027/Z000115</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop,mouse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop Lenovo ThinkPad EDGE E570</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PF0NG272</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 10.04.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150000029/Z000114</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workstation, Монитор Lenovo ThinkVision T2424z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workstation Lenovo ThinkStation P310</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S4BP0247</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New_поставить на учет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AiO, mouse, keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AiO Acer Aspire C24-2(U)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DQBRRCD00255101AA36N02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 16.07.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DQBRRCD00255101A546N02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">не на балансе_ИТ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop Lenovo t440p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC00V9QJ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 13.05.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop Lenovo T480</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PF1LY4VK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 20.08.2026
+Акт 16.09.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">поставить на учет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lenovo ThinkBook 16 G7 ARP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PW0K0D8T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DQBR8CD00255101D126N02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 18.05.2026</t>
   </si>
   <si>
     <t xml:space="preserve">вапифащгп ш</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AiO Acer Aspire C24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 18.11.2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
-    <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
+    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="168" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -112,8 +229,51 @@
       <family val="1"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -129,11 +289,35 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FF993300"/>
+        <bgColor rgb="FF9C0006"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0E0E3"/>
+        <bgColor rgb="FFCCCCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFF99"/>
+        <bgColor rgb="FFFFFF99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF969696"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
+        <bgColor rgb="FF33CCCC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -146,6 +330,29 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -174,7 +381,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -203,7 +410,95 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -216,6 +511,120 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -226,13 +635,13 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF9C0006"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFCCCCCC"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -241,7 +650,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFD0E0E3"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -252,15 +661,15 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFCCFF99"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFC7CE"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FF92D050"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -285,14 +694,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>798480</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>43560</xdr:rowOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>72360</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>386640</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>175320</xdr:rowOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>252000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -335,14 +744,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>798480</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>43560</xdr:rowOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>72360</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>386640</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>175320</xdr:rowOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>198720</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -564,7 +973,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1048576"/>
+  <dimension ref="A1:XFD1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.39"/>
@@ -610,27 +1019,1444 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="7" t="n">
+      <c r="C2" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="12"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="13"/>
+      <c r="W2" s="13"/>
+      <c r="X2" s="13"/>
+      <c r="Y2" s="13"/>
+      <c r="Z2" s="13"/>
+      <c r="AA2" s="13"/>
+      <c r="AB2" s="13"/>
+      <c r="AC2" s="13"/>
+      <c r="AD2" s="13"/>
+      <c r="AE2" s="13"/>
+      <c r="AF2" s="13"/>
+      <c r="AG2" s="13"/>
+      <c r="AH2" s="13"/>
+      <c r="AI2" s="13"/>
+      <c r="AJ2" s="13"/>
+      <c r="AK2" s="13"/>
+      <c r="AL2" s="13"/>
+      <c r="AM2" s="13"/>
+      <c r="AN2" s="13"/>
+      <c r="AO2" s="13"/>
+      <c r="AP2" s="13"/>
+      <c r="AQ2" s="13"/>
+      <c r="AR2" s="13"/>
+      <c r="AS2" s="13"/>
+      <c r="AT2" s="13"/>
+      <c r="AU2" s="13"/>
+      <c r="AV2" s="13"/>
+      <c r="AW2" s="13"/>
+      <c r="AX2" s="13"/>
+      <c r="AY2" s="13"/>
+      <c r="AZ2" s="13"/>
+      <c r="BA2" s="13"/>
+      <c r="BB2" s="13"/>
+      <c r="BC2" s="13"/>
+      <c r="BD2" s="13"/>
+      <c r="BE2" s="13"/>
+      <c r="BF2" s="13"/>
+      <c r="BG2" s="13"/>
+      <c r="BH2" s="13"/>
+      <c r="BI2" s="13"/>
+      <c r="BJ2" s="13"/>
+      <c r="BK2" s="13"/>
+      <c r="BL2" s="13"/>
+      <c r="BM2" s="13"/>
+      <c r="BN2" s="13"/>
+      <c r="BO2" s="13"/>
+      <c r="BP2" s="13"/>
+      <c r="BQ2" s="13"/>
+      <c r="BR2" s="13"/>
+      <c r="BS2" s="13"/>
+      <c r="BT2" s="13"/>
+      <c r="BU2" s="13"/>
+      <c r="BV2" s="13"/>
+      <c r="BW2" s="13"/>
+      <c r="BX2" s="13"/>
+      <c r="BY2" s="13"/>
+      <c r="BZ2" s="13"/>
+      <c r="CA2" s="13"/>
+      <c r="CB2" s="13"/>
+      <c r="CC2" s="13"/>
+      <c r="CD2" s="13"/>
+      <c r="CE2" s="13"/>
+      <c r="CF2" s="13"/>
+      <c r="CG2" s="13"/>
+      <c r="CH2" s="13"/>
+      <c r="CI2" s="13"/>
+      <c r="CJ2" s="13"/>
+      <c r="CK2" s="13"/>
+      <c r="CL2" s="13"/>
+      <c r="CM2" s="13"/>
+      <c r="CN2" s="13"/>
+      <c r="CO2" s="13"/>
+      <c r="CP2" s="13"/>
+      <c r="CQ2" s="13"/>
+      <c r="CR2" s="13"/>
+      <c r="CS2" s="13"/>
+      <c r="CT2" s="13"/>
+      <c r="CU2" s="13"/>
+      <c r="CV2" s="13"/>
+      <c r="CW2" s="13"/>
+      <c r="CX2" s="13"/>
+      <c r="CY2" s="13"/>
+      <c r="CZ2" s="13"/>
+      <c r="DA2" s="13"/>
+      <c r="DB2" s="13"/>
+      <c r="DC2" s="13"/>
+      <c r="DD2" s="13"/>
+      <c r="DE2" s="13"/>
+      <c r="DF2" s="13"/>
+      <c r="DG2" s="13"/>
+      <c r="DH2" s="13"/>
+      <c r="DI2" s="13"/>
+      <c r="DJ2" s="13"/>
+      <c r="DK2" s="13"/>
+      <c r="DL2" s="13"/>
+      <c r="DM2" s="13"/>
+      <c r="XFD2" s="0"/>
+    </row>
+    <row r="3" customFormat="false" ht="54.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="12"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="1"/>
+      <c r="W3" s="1"/>
+      <c r="X3" s="1"/>
+      <c r="Y3" s="1"/>
+      <c r="Z3" s="1"/>
+      <c r="AA3" s="1"/>
+      <c r="AB3" s="1"/>
+      <c r="AC3" s="1"/>
+      <c r="AD3" s="1"/>
+      <c r="AE3" s="1"/>
+      <c r="AF3" s="1"/>
+      <c r="AG3" s="1"/>
+      <c r="AH3" s="1"/>
+      <c r="AI3" s="1"/>
+      <c r="AJ3" s="1"/>
+      <c r="AK3" s="1"/>
+      <c r="AL3" s="1"/>
+      <c r="AM3" s="1"/>
+      <c r="AN3" s="1"/>
+      <c r="AO3" s="1"/>
+      <c r="AP3" s="1"/>
+      <c r="AQ3" s="1"/>
+      <c r="AR3" s="1"/>
+      <c r="AS3" s="1"/>
+      <c r="AT3" s="1"/>
+      <c r="AU3" s="1"/>
+      <c r="AV3" s="1"/>
+      <c r="AW3" s="1"/>
+      <c r="AX3" s="1"/>
+      <c r="AY3" s="1"/>
+      <c r="AZ3" s="1"/>
+      <c r="BA3" s="1"/>
+      <c r="BB3" s="1"/>
+      <c r="BC3" s="1"/>
+      <c r="BD3" s="1"/>
+      <c r="BE3" s="1"/>
+      <c r="BF3" s="1"/>
+      <c r="BG3" s="1"/>
+      <c r="BH3" s="1"/>
+      <c r="BI3" s="1"/>
+      <c r="BJ3" s="1"/>
+      <c r="BK3" s="1"/>
+      <c r="BL3" s="1"/>
+      <c r="BM3" s="1"/>
+      <c r="BN3" s="1"/>
+      <c r="BO3" s="1"/>
+      <c r="BP3" s="1"/>
+      <c r="BQ3" s="1"/>
+      <c r="BR3" s="1"/>
+      <c r="BS3" s="1"/>
+      <c r="BT3" s="1"/>
+      <c r="BU3" s="1"/>
+      <c r="BV3" s="1"/>
+      <c r="BW3" s="1"/>
+      <c r="BX3" s="1"/>
+      <c r="BY3" s="1"/>
+      <c r="BZ3" s="1"/>
+      <c r="CA3" s="1"/>
+      <c r="CB3" s="1"/>
+      <c r="CC3" s="1"/>
+      <c r="CD3" s="1"/>
+      <c r="CE3" s="1"/>
+      <c r="CF3" s="1"/>
+      <c r="CG3" s="1"/>
+      <c r="CH3" s="1"/>
+      <c r="CI3" s="1"/>
+      <c r="CJ3" s="1"/>
+      <c r="CK3" s="1"/>
+      <c r="CL3" s="1"/>
+      <c r="CM3" s="1"/>
+      <c r="CN3" s="1"/>
+      <c r="CO3" s="1"/>
+      <c r="CP3" s="1"/>
+      <c r="CQ3" s="1"/>
+      <c r="CR3" s="1"/>
+      <c r="CS3" s="1"/>
+      <c r="CT3" s="1"/>
+      <c r="CU3" s="1"/>
+      <c r="CV3" s="1"/>
+      <c r="CW3" s="1"/>
+      <c r="CX3" s="1"/>
+      <c r="CY3" s="1"/>
+      <c r="CZ3" s="1"/>
+      <c r="DA3" s="1"/>
+      <c r="DB3" s="1"/>
+      <c r="DC3" s="1"/>
+      <c r="DD3" s="1"/>
+      <c r="DE3" s="1"/>
+      <c r="DF3" s="1"/>
+      <c r="DG3" s="1"/>
+      <c r="DH3" s="1"/>
+      <c r="DI3" s="1"/>
+      <c r="DJ3" s="1"/>
+      <c r="DK3" s="1"/>
+      <c r="DL3" s="1"/>
+      <c r="DM3" s="1"/>
+      <c r="XFD3" s="0"/>
+    </row>
+    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="17"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="18"/>
+      <c r="R4" s="18"/>
+      <c r="S4" s="18"/>
+      <c r="T4" s="18"/>
+      <c r="U4" s="18"/>
+      <c r="V4" s="18"/>
+      <c r="W4" s="18"/>
+      <c r="X4" s="18"/>
+      <c r="Y4" s="18"/>
+      <c r="Z4" s="18"/>
+      <c r="AA4" s="18"/>
+      <c r="AB4" s="18"/>
+      <c r="AC4" s="18"/>
+      <c r="AD4" s="18"/>
+      <c r="AE4" s="18"/>
+      <c r="AF4" s="18"/>
+      <c r="AG4" s="18"/>
+      <c r="AH4" s="18"/>
+      <c r="AI4" s="18"/>
+      <c r="AJ4" s="18"/>
+      <c r="AK4" s="18"/>
+      <c r="AL4" s="18"/>
+      <c r="AM4" s="18"/>
+      <c r="AN4" s="18"/>
+      <c r="AO4" s="18"/>
+      <c r="AP4" s="18"/>
+      <c r="AQ4" s="18"/>
+      <c r="AR4" s="18"/>
+      <c r="AS4" s="18"/>
+      <c r="AT4" s="18"/>
+      <c r="AU4" s="18"/>
+      <c r="AV4" s="18"/>
+      <c r="AW4" s="18"/>
+      <c r="AX4" s="18"/>
+      <c r="AY4" s="18"/>
+      <c r="AZ4" s="18"/>
+      <c r="BA4" s="18"/>
+      <c r="BB4" s="18"/>
+      <c r="BC4" s="18"/>
+      <c r="BD4" s="18"/>
+      <c r="BE4" s="18"/>
+      <c r="BF4" s="18"/>
+      <c r="BG4" s="18"/>
+      <c r="BH4" s="18"/>
+      <c r="BI4" s="18"/>
+      <c r="BJ4" s="18"/>
+      <c r="BK4" s="18"/>
+      <c r="BL4" s="18"/>
+      <c r="BM4" s="18"/>
+      <c r="BN4" s="18"/>
+      <c r="BO4" s="18"/>
+      <c r="BP4" s="18"/>
+      <c r="BQ4" s="18"/>
+      <c r="BR4" s="18"/>
+      <c r="BS4" s="18"/>
+      <c r="BT4" s="18"/>
+      <c r="BU4" s="18"/>
+      <c r="BV4" s="18"/>
+      <c r="BW4" s="18"/>
+      <c r="BX4" s="18"/>
+      <c r="BY4" s="18"/>
+      <c r="BZ4" s="18"/>
+      <c r="CA4" s="18"/>
+      <c r="CB4" s="18"/>
+      <c r="CC4" s="18"/>
+      <c r="CD4" s="18"/>
+      <c r="CE4" s="18"/>
+      <c r="CF4" s="18"/>
+      <c r="CG4" s="18"/>
+      <c r="CH4" s="18"/>
+      <c r="CI4" s="18"/>
+      <c r="CJ4" s="18"/>
+      <c r="CK4" s="18"/>
+      <c r="CL4" s="18"/>
+      <c r="CM4" s="18"/>
+      <c r="CN4" s="18"/>
+      <c r="CO4" s="18"/>
+      <c r="CP4" s="18"/>
+      <c r="CQ4" s="18"/>
+      <c r="CR4" s="18"/>
+      <c r="CS4" s="18"/>
+      <c r="CT4" s="18"/>
+      <c r="CU4" s="18"/>
+      <c r="CV4" s="18"/>
+      <c r="CW4" s="18"/>
+      <c r="CX4" s="18"/>
+      <c r="CY4" s="18"/>
+      <c r="CZ4" s="18"/>
+      <c r="DA4" s="18"/>
+      <c r="DB4" s="18"/>
+      <c r="DC4" s="18"/>
+      <c r="DD4" s="18"/>
+      <c r="DE4" s="18"/>
+      <c r="DF4" s="18"/>
+      <c r="DG4" s="18"/>
+      <c r="DH4" s="18"/>
+      <c r="DI4" s="18"/>
+      <c r="DJ4" s="18"/>
+      <c r="DK4" s="18"/>
+      <c r="DL4" s="18"/>
+      <c r="DM4" s="18"/>
+      <c r="XFD4" s="0"/>
+    </row>
+    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>45510</v>
+      </c>
+      <c r="F5" s="12"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
+      <c r="Q5" s="13"/>
+      <c r="R5" s="13"/>
+      <c r="S5" s="13"/>
+      <c r="T5" s="13"/>
+      <c r="U5" s="13"/>
+      <c r="V5" s="13"/>
+      <c r="W5" s="13"/>
+      <c r="X5" s="13"/>
+      <c r="Y5" s="13"/>
+      <c r="Z5" s="13"/>
+      <c r="AA5" s="13"/>
+      <c r="AB5" s="13"/>
+      <c r="AC5" s="13"/>
+      <c r="AD5" s="13"/>
+      <c r="AE5" s="13"/>
+      <c r="AF5" s="13"/>
+      <c r="AG5" s="13"/>
+      <c r="AH5" s="13"/>
+      <c r="AI5" s="13"/>
+      <c r="AJ5" s="13"/>
+      <c r="AK5" s="13"/>
+      <c r="AL5" s="13"/>
+      <c r="AM5" s="13"/>
+      <c r="AN5" s="13"/>
+      <c r="AO5" s="13"/>
+      <c r="AP5" s="13"/>
+      <c r="AQ5" s="13"/>
+      <c r="AR5" s="13"/>
+      <c r="AS5" s="13"/>
+      <c r="AT5" s="13"/>
+      <c r="AU5" s="13"/>
+      <c r="AV5" s="13"/>
+      <c r="AW5" s="13"/>
+      <c r="AX5" s="13"/>
+      <c r="AY5" s="13"/>
+      <c r="AZ5" s="13"/>
+      <c r="BA5" s="13"/>
+      <c r="BB5" s="13"/>
+      <c r="BC5" s="13"/>
+      <c r="BD5" s="13"/>
+      <c r="BE5" s="13"/>
+      <c r="BF5" s="13"/>
+      <c r="BG5" s="13"/>
+      <c r="BH5" s="13"/>
+      <c r="BI5" s="13"/>
+      <c r="BJ5" s="13"/>
+      <c r="BK5" s="13"/>
+      <c r="BL5" s="13"/>
+      <c r="BM5" s="13"/>
+      <c r="BN5" s="13"/>
+      <c r="BO5" s="13"/>
+      <c r="BP5" s="13"/>
+      <c r="BQ5" s="13"/>
+      <c r="BR5" s="13"/>
+      <c r="BS5" s="13"/>
+      <c r="BT5" s="13"/>
+      <c r="BU5" s="13"/>
+      <c r="BV5" s="13"/>
+      <c r="BW5" s="13"/>
+      <c r="BX5" s="13"/>
+      <c r="BY5" s="13"/>
+      <c r="BZ5" s="13"/>
+      <c r="CA5" s="13"/>
+      <c r="CB5" s="13"/>
+      <c r="CC5" s="13"/>
+      <c r="CD5" s="13"/>
+      <c r="CE5" s="13"/>
+      <c r="CF5" s="13"/>
+      <c r="CG5" s="13"/>
+      <c r="CH5" s="13"/>
+      <c r="CI5" s="13"/>
+      <c r="CJ5" s="13"/>
+      <c r="CK5" s="13"/>
+      <c r="CL5" s="13"/>
+      <c r="CM5" s="13"/>
+      <c r="CN5" s="13"/>
+      <c r="CO5" s="13"/>
+      <c r="CP5" s="13"/>
+      <c r="CQ5" s="13"/>
+      <c r="CR5" s="13"/>
+      <c r="CS5" s="13"/>
+      <c r="CT5" s="13"/>
+      <c r="CU5" s="13"/>
+      <c r="CV5" s="13"/>
+      <c r="CW5" s="13"/>
+      <c r="CX5" s="13"/>
+      <c r="CY5" s="13"/>
+      <c r="CZ5" s="13"/>
+      <c r="DA5" s="13"/>
+      <c r="DB5" s="13"/>
+      <c r="DC5" s="13"/>
+      <c r="DD5" s="13"/>
+      <c r="DE5" s="13"/>
+      <c r="DF5" s="13"/>
+      <c r="DG5" s="13"/>
+      <c r="DH5" s="13"/>
+      <c r="DI5" s="13"/>
+      <c r="DJ5" s="13"/>
+      <c r="DK5" s="13"/>
+      <c r="DL5" s="13"/>
+      <c r="DM5" s="13"/>
+      <c r="XFD5" s="0"/>
+    </row>
+    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>46111</v>
+      </c>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="18"/>
+      <c r="T6" s="18"/>
+      <c r="U6" s="18"/>
+      <c r="V6" s="18"/>
+      <c r="W6" s="18"/>
+      <c r="X6" s="18"/>
+      <c r="Y6" s="18"/>
+      <c r="Z6" s="18"/>
+      <c r="AA6" s="18"/>
+      <c r="AB6" s="18"/>
+      <c r="AC6" s="18"/>
+      <c r="AD6" s="18"/>
+      <c r="AE6" s="18"/>
+      <c r="AF6" s="18"/>
+      <c r="AG6" s="18"/>
+      <c r="AH6" s="18"/>
+      <c r="AI6" s="18"/>
+      <c r="AJ6" s="18"/>
+      <c r="AK6" s="18"/>
+      <c r="AL6" s="18"/>
+      <c r="AM6" s="18"/>
+      <c r="AN6" s="18"/>
+      <c r="AO6" s="18"/>
+      <c r="AP6" s="18"/>
+      <c r="AQ6" s="18"/>
+      <c r="AR6" s="18"/>
+      <c r="AS6" s="18"/>
+      <c r="AT6" s="18"/>
+      <c r="AU6" s="18"/>
+      <c r="AV6" s="18"/>
+      <c r="AW6" s="18"/>
+      <c r="AX6" s="18"/>
+      <c r="AY6" s="18"/>
+      <c r="AZ6" s="18"/>
+      <c r="BA6" s="18"/>
+      <c r="BB6" s="18"/>
+      <c r="BC6" s="18"/>
+      <c r="BD6" s="18"/>
+      <c r="BE6" s="18"/>
+      <c r="BF6" s="18"/>
+      <c r="BG6" s="18"/>
+      <c r="BH6" s="18"/>
+      <c r="BI6" s="18"/>
+      <c r="BJ6" s="18"/>
+      <c r="BK6" s="18"/>
+      <c r="BL6" s="18"/>
+      <c r="BM6" s="18"/>
+      <c r="BN6" s="18"/>
+      <c r="BO6" s="18"/>
+      <c r="BP6" s="18"/>
+      <c r="BQ6" s="18"/>
+      <c r="BR6" s="18"/>
+      <c r="BS6" s="18"/>
+      <c r="BT6" s="18"/>
+      <c r="BU6" s="18"/>
+      <c r="BV6" s="18"/>
+      <c r="BW6" s="18"/>
+      <c r="BX6" s="18"/>
+      <c r="BY6" s="18"/>
+      <c r="BZ6" s="18"/>
+      <c r="CA6" s="18"/>
+      <c r="CB6" s="18"/>
+      <c r="CC6" s="18"/>
+      <c r="CD6" s="18"/>
+      <c r="CE6" s="18"/>
+      <c r="CF6" s="18"/>
+      <c r="CG6" s="18"/>
+      <c r="CH6" s="18"/>
+      <c r="CI6" s="18"/>
+      <c r="CJ6" s="18"/>
+      <c r="CK6" s="18"/>
+      <c r="CL6" s="18"/>
+      <c r="CM6" s="18"/>
+      <c r="CN6" s="18"/>
+      <c r="CO6" s="18"/>
+      <c r="CP6" s="18"/>
+      <c r="CQ6" s="18"/>
+      <c r="CR6" s="18"/>
+      <c r="CS6" s="18"/>
+      <c r="CT6" s="18"/>
+      <c r="CU6" s="18"/>
+      <c r="CV6" s="18"/>
+      <c r="CW6" s="18"/>
+      <c r="CX6" s="18"/>
+      <c r="CY6" s="18"/>
+      <c r="CZ6" s="18"/>
+      <c r="DA6" s="18"/>
+      <c r="DB6" s="18"/>
+      <c r="DC6" s="18"/>
+      <c r="DD6" s="18"/>
+      <c r="DE6" s="18"/>
+      <c r="DF6" s="18"/>
+      <c r="DG6" s="18"/>
+      <c r="DH6" s="18"/>
+      <c r="DI6" s="18"/>
+      <c r="DJ6" s="18"/>
+      <c r="DK6" s="18"/>
+      <c r="DL6" s="18"/>
+      <c r="DM6" s="18"/>
+      <c r="XFD6" s="0"/>
+    </row>
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>46111</v>
+      </c>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="13"/>
+      <c r="Q7" s="13"/>
+      <c r="R7" s="13"/>
+      <c r="S7" s="13"/>
+      <c r="T7" s="13"/>
+      <c r="U7" s="13"/>
+      <c r="V7" s="13"/>
+      <c r="W7" s="13"/>
+      <c r="X7" s="13"/>
+      <c r="Y7" s="13"/>
+      <c r="Z7" s="13"/>
+      <c r="AA7" s="13"/>
+      <c r="AB7" s="13"/>
+      <c r="AC7" s="13"/>
+      <c r="AD7" s="13"/>
+      <c r="AE7" s="13"/>
+      <c r="AF7" s="13"/>
+      <c r="AG7" s="13"/>
+      <c r="AH7" s="13"/>
+      <c r="AI7" s="13"/>
+      <c r="AJ7" s="13"/>
+      <c r="AK7" s="13"/>
+      <c r="AL7" s="13"/>
+      <c r="AM7" s="13"/>
+      <c r="AN7" s="13"/>
+      <c r="AO7" s="13"/>
+      <c r="AP7" s="13"/>
+      <c r="AQ7" s="13"/>
+      <c r="AR7" s="13"/>
+      <c r="AS7" s="13"/>
+      <c r="AT7" s="13"/>
+      <c r="AU7" s="13"/>
+      <c r="AV7" s="13"/>
+      <c r="AW7" s="13"/>
+      <c r="AX7" s="13"/>
+      <c r="AY7" s="13"/>
+      <c r="AZ7" s="13"/>
+      <c r="BA7" s="13"/>
+      <c r="BB7" s="13"/>
+      <c r="BC7" s="13"/>
+      <c r="BD7" s="13"/>
+      <c r="BE7" s="13"/>
+      <c r="BF7" s="13"/>
+      <c r="BG7" s="13"/>
+      <c r="BH7" s="13"/>
+      <c r="BI7" s="13"/>
+      <c r="BJ7" s="13"/>
+      <c r="BK7" s="13"/>
+      <c r="BL7" s="13"/>
+      <c r="BM7" s="13"/>
+      <c r="BN7" s="13"/>
+      <c r="BO7" s="13"/>
+      <c r="BP7" s="13"/>
+      <c r="BQ7" s="13"/>
+      <c r="BR7" s="13"/>
+      <c r="BS7" s="13"/>
+      <c r="BT7" s="13"/>
+      <c r="BU7" s="13"/>
+      <c r="BV7" s="13"/>
+      <c r="BW7" s="13"/>
+      <c r="BX7" s="13"/>
+      <c r="BY7" s="13"/>
+      <c r="BZ7" s="13"/>
+      <c r="CA7" s="13"/>
+      <c r="CB7" s="13"/>
+      <c r="CC7" s="13"/>
+      <c r="CD7" s="13"/>
+      <c r="CE7" s="13"/>
+      <c r="CF7" s="13"/>
+      <c r="CG7" s="13"/>
+      <c r="CH7" s="13"/>
+      <c r="CI7" s="13"/>
+      <c r="CJ7" s="13"/>
+      <c r="CK7" s="13"/>
+      <c r="CL7" s="13"/>
+      <c r="CM7" s="13"/>
+      <c r="CN7" s="13"/>
+      <c r="CO7" s="13"/>
+      <c r="CP7" s="13"/>
+      <c r="CQ7" s="13"/>
+      <c r="CR7" s="13"/>
+      <c r="CS7" s="13"/>
+      <c r="CT7" s="13"/>
+      <c r="CU7" s="13"/>
+      <c r="CV7" s="13"/>
+      <c r="CW7" s="13"/>
+      <c r="CX7" s="13"/>
+      <c r="CY7" s="13"/>
+      <c r="CZ7" s="13"/>
+      <c r="DA7" s="13"/>
+      <c r="DB7" s="13"/>
+      <c r="DC7" s="13"/>
+      <c r="DD7" s="13"/>
+      <c r="DE7" s="13"/>
+      <c r="DF7" s="13"/>
+      <c r="DG7" s="13"/>
+      <c r="DH7" s="13"/>
+      <c r="DI7" s="13"/>
+      <c r="DJ7" s="13"/>
+      <c r="DK7" s="13"/>
+      <c r="DL7" s="13"/>
+      <c r="DM7" s="13"/>
+      <c r="XFD7" s="0"/>
+    </row>
+    <row r="8" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="21"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="22"/>
+      <c r="R8" s="22"/>
+      <c r="S8" s="22"/>
+      <c r="T8" s="22"/>
+      <c r="U8" s="22"/>
+      <c r="V8" s="22"/>
+      <c r="W8" s="22"/>
+      <c r="X8" s="22"/>
+      <c r="Y8" s="22"/>
+      <c r="Z8" s="22"/>
+      <c r="AA8" s="22"/>
+      <c r="AB8" s="22"/>
+      <c r="AC8" s="22"/>
+      <c r="AD8" s="22"/>
+      <c r="AE8" s="22"/>
+      <c r="AF8" s="22"/>
+      <c r="AG8" s="22"/>
+      <c r="AH8" s="22"/>
+      <c r="AI8" s="22"/>
+      <c r="AJ8" s="22"/>
+      <c r="AK8" s="22"/>
+      <c r="AL8" s="22"/>
+      <c r="AM8" s="22"/>
+      <c r="AN8" s="22"/>
+      <c r="AO8" s="22"/>
+      <c r="AP8" s="22"/>
+      <c r="AQ8" s="22"/>
+      <c r="AR8" s="22"/>
+      <c r="AS8" s="22"/>
+      <c r="AT8" s="22"/>
+      <c r="AU8" s="22"/>
+      <c r="AV8" s="22"/>
+      <c r="AW8" s="22"/>
+      <c r="AX8" s="22"/>
+      <c r="AY8" s="22"/>
+      <c r="AZ8" s="22"/>
+      <c r="BA8" s="22"/>
+      <c r="BB8" s="22"/>
+      <c r="BC8" s="22"/>
+      <c r="BD8" s="22"/>
+      <c r="BE8" s="22"/>
+      <c r="BF8" s="22"/>
+      <c r="BG8" s="22"/>
+      <c r="BH8" s="22"/>
+      <c r="BI8" s="22"/>
+      <c r="BJ8" s="22"/>
+      <c r="BK8" s="22"/>
+      <c r="BL8" s="22"/>
+      <c r="BM8" s="22"/>
+      <c r="BN8" s="22"/>
+      <c r="BO8" s="22"/>
+      <c r="BP8" s="22"/>
+      <c r="BQ8" s="22"/>
+      <c r="BR8" s="22"/>
+      <c r="BS8" s="22"/>
+      <c r="BT8" s="22"/>
+      <c r="BU8" s="22"/>
+      <c r="BV8" s="22"/>
+      <c r="BW8" s="22"/>
+      <c r="BX8" s="22"/>
+      <c r="BY8" s="22"/>
+      <c r="BZ8" s="22"/>
+      <c r="CA8" s="22"/>
+      <c r="CB8" s="22"/>
+      <c r="CC8" s="22"/>
+      <c r="CD8" s="22"/>
+      <c r="CE8" s="22"/>
+      <c r="CF8" s="22"/>
+      <c r="CG8" s="22"/>
+      <c r="CH8" s="22"/>
+      <c r="CI8" s="22"/>
+      <c r="CJ8" s="22"/>
+      <c r="CK8" s="22"/>
+      <c r="CL8" s="22"/>
+      <c r="CM8" s="22"/>
+      <c r="CN8" s="22"/>
+      <c r="CO8" s="22"/>
+      <c r="CP8" s="22"/>
+      <c r="CQ8" s="22"/>
+      <c r="CR8" s="22"/>
+      <c r="CS8" s="22"/>
+      <c r="CT8" s="22"/>
+      <c r="CU8" s="22"/>
+      <c r="CV8" s="22"/>
+      <c r="CW8" s="22"/>
+      <c r="CX8" s="22"/>
+      <c r="CY8" s="22"/>
+      <c r="CZ8" s="22"/>
+      <c r="DA8" s="22"/>
+      <c r="DB8" s="22"/>
+      <c r="DC8" s="22"/>
+      <c r="DD8" s="22"/>
+      <c r="DE8" s="22"/>
+      <c r="DF8" s="22"/>
+      <c r="DG8" s="22"/>
+      <c r="DH8" s="22"/>
+      <c r="DI8" s="22"/>
+      <c r="DJ8" s="22"/>
+      <c r="DK8" s="22"/>
+      <c r="DL8" s="22"/>
+      <c r="DM8" s="22"/>
+      <c r="XFD8" s="0"/>
+    </row>
+    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
+      <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18"/>
+      <c r="R9" s="18"/>
+      <c r="S9" s="18"/>
+      <c r="T9" s="18"/>
+      <c r="U9" s="18"/>
+      <c r="V9" s="18"/>
+      <c r="W9" s="18"/>
+      <c r="X9" s="18"/>
+      <c r="Y9" s="18"/>
+      <c r="Z9" s="18"/>
+      <c r="AA9" s="18"/>
+      <c r="AB9" s="18"/>
+      <c r="AC9" s="18"/>
+      <c r="AD9" s="18"/>
+      <c r="AE9" s="18"/>
+      <c r="AF9" s="18"/>
+      <c r="AG9" s="18"/>
+      <c r="AH9" s="18"/>
+      <c r="AI9" s="18"/>
+      <c r="AJ9" s="18"/>
+      <c r="AK9" s="18"/>
+      <c r="AL9" s="18"/>
+      <c r="AM9" s="18"/>
+      <c r="AN9" s="18"/>
+      <c r="AO9" s="18"/>
+      <c r="AP9" s="18"/>
+      <c r="AQ9" s="18"/>
+      <c r="AR9" s="18"/>
+      <c r="AS9" s="18"/>
+      <c r="AT9" s="18"/>
+      <c r="AU9" s="18"/>
+      <c r="AV9" s="18"/>
+      <c r="AW9" s="18"/>
+      <c r="AX9" s="18"/>
+      <c r="AY9" s="18"/>
+      <c r="AZ9" s="18"/>
+      <c r="BA9" s="18"/>
+      <c r="BB9" s="18"/>
+      <c r="BC9" s="18"/>
+      <c r="BD9" s="18"/>
+      <c r="BE9" s="18"/>
+      <c r="BF9" s="18"/>
+      <c r="BG9" s="18"/>
+      <c r="BH9" s="18"/>
+      <c r="BI9" s="18"/>
+      <c r="BJ9" s="18"/>
+      <c r="BK9" s="18"/>
+      <c r="BL9" s="18"/>
+      <c r="BM9" s="18"/>
+      <c r="BN9" s="18"/>
+      <c r="BO9" s="18"/>
+      <c r="BP9" s="18"/>
+      <c r="BQ9" s="18"/>
+      <c r="BR9" s="18"/>
+      <c r="BS9" s="18"/>
+      <c r="BT9" s="18"/>
+      <c r="BU9" s="18"/>
+      <c r="BV9" s="18"/>
+      <c r="BW9" s="18"/>
+      <c r="BX9" s="18"/>
+      <c r="BY9" s="18"/>
+      <c r="BZ9" s="18"/>
+      <c r="CA9" s="18"/>
+      <c r="CB9" s="18"/>
+      <c r="CC9" s="18"/>
+      <c r="CD9" s="18"/>
+      <c r="CE9" s="18"/>
+      <c r="CF9" s="18"/>
+      <c r="CG9" s="18"/>
+      <c r="CH9" s="18"/>
+      <c r="CI9" s="18"/>
+      <c r="CJ9" s="18"/>
+      <c r="CK9" s="18"/>
+      <c r="CL9" s="18"/>
+      <c r="CM9" s="18"/>
+      <c r="CN9" s="18"/>
+      <c r="CO9" s="18"/>
+      <c r="CP9" s="18"/>
+      <c r="CQ9" s="18"/>
+      <c r="CR9" s="18"/>
+      <c r="CS9" s="18"/>
+      <c r="CT9" s="18"/>
+      <c r="CU9" s="18"/>
+      <c r="CV9" s="18"/>
+      <c r="CW9" s="18"/>
+      <c r="CX9" s="18"/>
+      <c r="CY9" s="18"/>
+      <c r="CZ9" s="18"/>
+      <c r="DA9" s="18"/>
+      <c r="DB9" s="18"/>
+      <c r="DC9" s="18"/>
+      <c r="DD9" s="18"/>
+      <c r="DE9" s="18"/>
+      <c r="DF9" s="18"/>
+      <c r="DG9" s="18"/>
+      <c r="DH9" s="18"/>
+      <c r="DI9" s="18"/>
+      <c r="DJ9" s="18"/>
+      <c r="DK9" s="18"/>
+      <c r="DL9" s="18"/>
+      <c r="DM9" s="18"/>
+      <c r="XFD9" s="0"/>
+    </row>
+    <row r="10" customFormat="false" ht="41.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="23"/>
+      <c r="F10" s="24" t="n">
+        <v>46122</v>
+      </c>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="13"/>
+      <c r="R10" s="13"/>
+      <c r="S10" s="13"/>
+      <c r="T10" s="13"/>
+      <c r="U10" s="13"/>
+      <c r="V10" s="13"/>
+      <c r="W10" s="13"/>
+      <c r="X10" s="13"/>
+      <c r="Y10" s="13"/>
+      <c r="Z10" s="13"/>
+      <c r="AA10" s="13"/>
+      <c r="AB10" s="13"/>
+      <c r="AC10" s="13"/>
+      <c r="AD10" s="13"/>
+      <c r="AE10" s="13"/>
+      <c r="AF10" s="13"/>
+      <c r="AG10" s="13"/>
+      <c r="AH10" s="13"/>
+      <c r="AI10" s="13"/>
+      <c r="AJ10" s="13"/>
+      <c r="AK10" s="13"/>
+      <c r="AL10" s="13"/>
+      <c r="AM10" s="13"/>
+      <c r="AN10" s="13"/>
+      <c r="AO10" s="13"/>
+      <c r="AP10" s="13"/>
+      <c r="AQ10" s="13"/>
+      <c r="AR10" s="13"/>
+      <c r="AS10" s="13"/>
+      <c r="AT10" s="13"/>
+      <c r="AU10" s="13"/>
+      <c r="AV10" s="13"/>
+      <c r="AW10" s="13"/>
+      <c r="AX10" s="13"/>
+      <c r="AY10" s="13"/>
+      <c r="AZ10" s="13"/>
+      <c r="BA10" s="13"/>
+      <c r="BB10" s="13"/>
+      <c r="BC10" s="13"/>
+      <c r="BD10" s="13"/>
+      <c r="BE10" s="13"/>
+      <c r="BF10" s="13"/>
+      <c r="BG10" s="13"/>
+      <c r="BH10" s="13"/>
+      <c r="BI10" s="13"/>
+      <c r="BJ10" s="13"/>
+      <c r="BK10" s="13"/>
+      <c r="BL10" s="13"/>
+      <c r="BM10" s="13"/>
+      <c r="BN10" s="13"/>
+      <c r="BO10" s="13"/>
+      <c r="BP10" s="13"/>
+      <c r="BQ10" s="13"/>
+      <c r="BR10" s="13"/>
+      <c r="BS10" s="13"/>
+      <c r="BT10" s="13"/>
+      <c r="BU10" s="13"/>
+      <c r="BV10" s="13"/>
+      <c r="BW10" s="13"/>
+      <c r="BX10" s="13"/>
+      <c r="BY10" s="13"/>
+      <c r="BZ10" s="13"/>
+      <c r="CA10" s="13"/>
+      <c r="CB10" s="13"/>
+      <c r="CC10" s="13"/>
+      <c r="CD10" s="13"/>
+      <c r="CE10" s="13"/>
+      <c r="CF10" s="13"/>
+      <c r="CG10" s="13"/>
+      <c r="CH10" s="13"/>
+      <c r="CI10" s="13"/>
+      <c r="CJ10" s="13"/>
+      <c r="CK10" s="13"/>
+      <c r="CL10" s="13"/>
+      <c r="CM10" s="13"/>
+      <c r="CN10" s="13"/>
+      <c r="CO10" s="13"/>
+      <c r="CP10" s="13"/>
+      <c r="CQ10" s="13"/>
+      <c r="CR10" s="13"/>
+      <c r="CS10" s="13"/>
+      <c r="CT10" s="13"/>
+      <c r="CU10" s="13"/>
+      <c r="CV10" s="13"/>
+      <c r="CW10" s="13"/>
+      <c r="CX10" s="13"/>
+      <c r="CY10" s="13"/>
+      <c r="CZ10" s="13"/>
+      <c r="DA10" s="13"/>
+      <c r="DB10" s="13"/>
+      <c r="DC10" s="13"/>
+      <c r="DD10" s="13"/>
+      <c r="DE10" s="13"/>
+      <c r="DF10" s="13"/>
+      <c r="DG10" s="13"/>
+      <c r="DH10" s="13"/>
+      <c r="DI10" s="13"/>
+      <c r="DJ10" s="13"/>
+      <c r="DK10" s="13"/>
+      <c r="DL10" s="13"/>
+      <c r="DM10" s="13"/>
+      <c r="XFD10" s="0"/>
+    </row>
+    <row r="11" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="21"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="28"/>
+      <c r="L11" s="28"/>
+      <c r="M11" s="28"/>
+      <c r="N11" s="28"/>
+      <c r="O11" s="28"/>
+      <c r="P11" s="28"/>
+      <c r="Q11" s="28"/>
+      <c r="R11" s="28"/>
+      <c r="S11" s="28"/>
+      <c r="T11" s="28"/>
+      <c r="U11" s="28"/>
+      <c r="V11" s="28"/>
+      <c r="W11" s="28"/>
+      <c r="X11" s="28"/>
+      <c r="Y11" s="28"/>
+      <c r="Z11" s="28"/>
+      <c r="AA11" s="28"/>
+      <c r="AB11" s="28"/>
+      <c r="AC11" s="28"/>
+      <c r="AD11" s="28"/>
+      <c r="AE11" s="28"/>
+      <c r="AF11" s="28"/>
+      <c r="AG11" s="28"/>
+      <c r="AH11" s="28"/>
+      <c r="AI11" s="28"/>
+      <c r="AJ11" s="28"/>
+      <c r="AK11" s="28"/>
+      <c r="AL11" s="28"/>
+      <c r="AM11" s="28"/>
+      <c r="AN11" s="28"/>
+      <c r="AO11" s="28"/>
+      <c r="AP11" s="28"/>
+      <c r="AQ11" s="28"/>
+      <c r="AR11" s="28"/>
+      <c r="AS11" s="28"/>
+      <c r="AT11" s="28"/>
+      <c r="AU11" s="28"/>
+      <c r="AV11" s="28"/>
+      <c r="AW11" s="28"/>
+      <c r="AX11" s="28"/>
+      <c r="AY11" s="28"/>
+      <c r="AZ11" s="28"/>
+      <c r="BA11" s="28"/>
+      <c r="BB11" s="28"/>
+      <c r="BC11" s="28"/>
+      <c r="BD11" s="28"/>
+      <c r="BE11" s="28"/>
+      <c r="BF11" s="28"/>
+      <c r="BG11" s="28"/>
+      <c r="BH11" s="28"/>
+      <c r="BI11" s="28"/>
+      <c r="BJ11" s="28"/>
+      <c r="BK11" s="28"/>
+      <c r="BL11" s="28"/>
+      <c r="BM11" s="28"/>
+      <c r="BN11" s="28"/>
+      <c r="BO11" s="28"/>
+      <c r="BP11" s="28"/>
+      <c r="BQ11" s="28"/>
+      <c r="BR11" s="28"/>
+      <c r="BS11" s="28"/>
+      <c r="BT11" s="28"/>
+      <c r="BU11" s="28"/>
+      <c r="BV11" s="28"/>
+      <c r="BW11" s="28"/>
+      <c r="BX11" s="28"/>
+      <c r="BY11" s="28"/>
+      <c r="BZ11" s="28"/>
+      <c r="CA11" s="28"/>
+      <c r="CB11" s="28"/>
+      <c r="CC11" s="28"/>
+      <c r="CD11" s="28"/>
+      <c r="CE11" s="28"/>
+      <c r="CF11" s="28"/>
+      <c r="CG11" s="28"/>
+      <c r="CH11" s="28"/>
+      <c r="CI11" s="28"/>
+      <c r="CJ11" s="28"/>
+      <c r="CK11" s="28"/>
+      <c r="CL11" s="28"/>
+      <c r="CM11" s="28"/>
+      <c r="CN11" s="28"/>
+      <c r="CO11" s="28"/>
+      <c r="CP11" s="28"/>
+      <c r="CQ11" s="28"/>
+      <c r="CR11" s="28"/>
+      <c r="CS11" s="28"/>
+      <c r="CT11" s="28"/>
+      <c r="CU11" s="28"/>
+      <c r="CV11" s="28"/>
+      <c r="CW11" s="28"/>
+      <c r="CX11" s="28"/>
+      <c r="CY11" s="28"/>
+      <c r="CZ11" s="28"/>
+      <c r="DA11" s="28"/>
+      <c r="DB11" s="28"/>
+      <c r="DC11" s="28"/>
+      <c r="DD11" s="28"/>
+      <c r="DE11" s="28"/>
+      <c r="DF11" s="28"/>
+      <c r="DG11" s="28"/>
+      <c r="DH11" s="28"/>
+      <c r="DI11" s="28"/>
+      <c r="DJ11" s="28"/>
+      <c r="DK11" s="28"/>
+      <c r="DL11" s="28"/>
+      <c r="DM11" s="28"/>
+      <c r="XFD11" s="0"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="29" t="n">
         <v>57483</v>
       </c>
     </row>
-    <row r="1048321" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048322" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048323" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048324" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048325" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048326" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048327" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048328" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048329" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048330" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="10"/>
+      <c r="E13" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F13" s="21"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="28"/>
+      <c r="K13" s="28"/>
+      <c r="L13" s="28"/>
+      <c r="M13" s="28"/>
+      <c r="N13" s="28"/>
+      <c r="O13" s="28"/>
+      <c r="P13" s="28"/>
+      <c r="Q13" s="28"/>
+      <c r="R13" s="28"/>
+      <c r="S13" s="28"/>
+      <c r="T13" s="28"/>
+      <c r="U13" s="28"/>
+      <c r="V13" s="28"/>
+      <c r="W13" s="28"/>
+      <c r="X13" s="28"/>
+      <c r="Y13" s="28"/>
+      <c r="Z13" s="28"/>
+      <c r="AA13" s="28"/>
+      <c r="AB13" s="28"/>
+      <c r="AC13" s="28"/>
+      <c r="AD13" s="28"/>
+      <c r="AE13" s="28"/>
+      <c r="AF13" s="28"/>
+      <c r="AG13" s="28"/>
+      <c r="AH13" s="28"/>
+      <c r="AI13" s="28"/>
+      <c r="AJ13" s="28"/>
+      <c r="AK13" s="28"/>
+      <c r="AL13" s="28"/>
+      <c r="AM13" s="28"/>
+      <c r="AN13" s="28"/>
+      <c r="AO13" s="28"/>
+      <c r="AP13" s="28"/>
+      <c r="AQ13" s="28"/>
+      <c r="AR13" s="28"/>
+      <c r="AS13" s="28"/>
+      <c r="AT13" s="28"/>
+      <c r="AU13" s="28"/>
+      <c r="AV13" s="28"/>
+      <c r="AW13" s="28"/>
+      <c r="AX13" s="28"/>
+      <c r="AY13" s="28"/>
+      <c r="AZ13" s="28"/>
+      <c r="BA13" s="28"/>
+      <c r="BB13" s="28"/>
+      <c r="BC13" s="28"/>
+      <c r="BD13" s="28"/>
+      <c r="BE13" s="28"/>
+      <c r="BF13" s="28"/>
+      <c r="BG13" s="28"/>
+      <c r="BH13" s="28"/>
+      <c r="BI13" s="28"/>
+      <c r="BJ13" s="28"/>
+      <c r="BK13" s="28"/>
+      <c r="BL13" s="28"/>
+      <c r="BM13" s="28"/>
+      <c r="BN13" s="28"/>
+      <c r="BO13" s="28"/>
+      <c r="BP13" s="28"/>
+      <c r="BQ13" s="28"/>
+      <c r="BR13" s="28"/>
+      <c r="BS13" s="28"/>
+      <c r="BT13" s="28"/>
+      <c r="BU13" s="28"/>
+      <c r="BV13" s="28"/>
+      <c r="BW13" s="28"/>
+      <c r="BX13" s="28"/>
+      <c r="BY13" s="28"/>
+      <c r="BZ13" s="28"/>
+      <c r="CA13" s="28"/>
+      <c r="CB13" s="28"/>
+      <c r="CC13" s="28"/>
+      <c r="CD13" s="28"/>
+      <c r="CE13" s="28"/>
+      <c r="CF13" s="28"/>
+      <c r="CG13" s="28"/>
+      <c r="CH13" s="28"/>
+      <c r="CI13" s="28"/>
+      <c r="CJ13" s="28"/>
+      <c r="CK13" s="28"/>
+      <c r="CL13" s="28"/>
+      <c r="CM13" s="28"/>
+      <c r="CN13" s="28"/>
+      <c r="CO13" s="28"/>
+      <c r="CP13" s="28"/>
+      <c r="CQ13" s="28"/>
+      <c r="CR13" s="28"/>
+      <c r="CS13" s="28"/>
+      <c r="CT13" s="28"/>
+      <c r="CU13" s="28"/>
+      <c r="CV13" s="28"/>
+      <c r="CW13" s="28"/>
+      <c r="CX13" s="28"/>
+      <c r="CY13" s="28"/>
+      <c r="CZ13" s="28"/>
+      <c r="DA13" s="28"/>
+      <c r="DB13" s="28"/>
+      <c r="DC13" s="28"/>
+      <c r="DD13" s="28"/>
+      <c r="DE13" s="28"/>
+      <c r="DF13" s="28"/>
+      <c r="DG13" s="28"/>
+      <c r="DH13" s="28"/>
+      <c r="DI13" s="28"/>
+      <c r="DJ13" s="28"/>
+      <c r="DK13" s="28"/>
+      <c r="DL13" s="28"/>
+      <c r="DM13" s="28"/>
+      <c r="XFD13" s="0"/>
+    </row>
     <row r="1048331" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048332" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048333" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -878,6 +2704,38 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
+  <conditionalFormatting sqref="B11 B13">
+    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="0">
+      <formula>NOT(ISERROR(SEARCH("workstation",B11)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10">
+    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="1">
+      <formula>NOT(ISERROR(SEARCH("workstation",B10)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4">
+    <cfRule type="containsText" priority="4" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="2">
+      <formula>NOT(ISERROR(SEARCH("workstation",B4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="5" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="3">
+      <formula>NOT(ISERROR(SEARCH("workstation",B4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="6" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="4">
+      <formula>NOT(ISERROR(SEARCH("workstation",B4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="7" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="5">
+      <formula>NOT(ISERROR(SEARCH("workstation",B4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="8" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="6">
+      <formula>NOT(ISERROR(SEARCH("workstation",B4)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2">
+    <cfRule type="containsText" priority="9" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="7">
+      <formula>NOT(ISERROR(SEARCH("workstation",B2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
delete computed_field for Asset.py
</commit_message>
<xml_diff>
--- a/xlsx/asset_import_template (2).xlsx
+++ b/xlsx/asset_import_template (2).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="49">
   <si>
     <t xml:space="preserve">Инвентарный номер / Inventory number</t>
   </si>
@@ -50,39 +50,139 @@
     <t xml:space="preserve">Период проверки / Check period</t>
   </si>
   <si>
-    <t xml:space="preserve">Laptop,mouse,bag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lenovo ThinkBook 15 G4 IAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MP2KDZYH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Акт 18.12.2024</t>
+    <t xml:space="preserve">140000257</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WorkStation,mouse,keyboard, monitor Lenovo 2424d ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workstation Lenovo ThinkStation P 320</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC10AS96</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 28.11.2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">140000420</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WorkStation,monitor(Lenovo T2324dC),mouse,keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рабочая станция Lenovo ThinkStation P310+монитор</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S4BP0263</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 14.08.2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150000027/Z000115</t>
   </si>
   <si>
     <t xml:space="preserve">Laptop,mouse</t>
   </si>
   <si>
-    <t xml:space="preserve">Laptop Acer Extensa 15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NXEGYER00H32008A5D3400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Акт 27.03.2026</t>
+    <t xml:space="preserve">Laptop Lenovo ThinkPad EDGE E570</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PF0NG272</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 10.04.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150000029/Z000114</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workstation, Монитор Lenovo ThinkVision T2424z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workstation Lenovo ThinkStation P310</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S4BP0247</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New_поставить на учет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AiO, mouse, keyboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AiO Acer Aspire C24-2(U)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DQBRRCD00255101AA36N02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 16.07.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DQBRRCD00255101A546N02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">не на балансе_ИТ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop Lenovo t440p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC00V9QJ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 13.05.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop Lenovo T480</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PF1LY4VK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 20.08.2026
+Акт 16.09.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">поставить на учет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lenovo ThinkBook 16 G7 ARP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PW0K0D8T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DQBR8CD00255101D126N02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 18.05.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вапифащгп ш</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AiO Acer Aspire C24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Акт 18.11.2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
+    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="168" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -138,14 +238,42 @@
       <charset val="204"/>
     </font>
     <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -161,13 +289,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FF993300"/>
+        <bgColor rgb="FF9C0006"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD0E0E3"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <bgColor rgb="FFCCCCCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -179,11 +307,17 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor rgb="FFC0C0C0"/>
+        <bgColor rgb="FF969696"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
+        <bgColor rgb="FF33CCCC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -196,6 +330,29 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -224,7 +381,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -257,11 +414,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -269,12 +434,72 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -286,6 +511,120 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF9C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -296,13 +635,13 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF9C0006"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFCCCCCC"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -327,7 +666,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFC7CE"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF92D050"/>
@@ -355,14 +694,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>798480</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>236160</xdr:rowOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>72360</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>644760</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>60120</xdr:rowOff>
+      <xdr:colOff>386640</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>252000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -372,7 +711,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="798480" y="927000"/>
-          <a:ext cx="9839880" cy="2990160"/>
+          <a:ext cx="9838800" cy="2989080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -405,14 +744,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>798480</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>236160</xdr:rowOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>72360</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>644760</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>60120</xdr:rowOff>
+      <xdr:colOff>386640</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>198720</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -422,7 +761,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="798480" y="927000"/>
-          <a:ext cx="9839880" cy="2228040"/>
+          <a:ext cx="9838800" cy="2226960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -634,11 +973,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1048576"/>
+  <dimension ref="A1:XFD1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.4"/>
@@ -651,7 +990,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="54.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -680,50 +1019,1529 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="41.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
-        <v>100000002700</v>
+    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>9</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="10"/>
+        <v>13</v>
+      </c>
+      <c r="F2" s="12"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="13"/>
+      <c r="W2" s="13"/>
+      <c r="X2" s="13"/>
+      <c r="Y2" s="13"/>
+      <c r="Z2" s="13"/>
+      <c r="AA2" s="13"/>
+      <c r="AB2" s="13"/>
+      <c r="AC2" s="13"/>
+      <c r="AD2" s="13"/>
+      <c r="AE2" s="13"/>
+      <c r="AF2" s="13"/>
+      <c r="AG2" s="13"/>
+      <c r="AH2" s="13"/>
+      <c r="AI2" s="13"/>
+      <c r="AJ2" s="13"/>
+      <c r="AK2" s="13"/>
+      <c r="AL2" s="13"/>
+      <c r="AM2" s="13"/>
+      <c r="AN2" s="13"/>
+      <c r="AO2" s="13"/>
+      <c r="AP2" s="13"/>
+      <c r="AQ2" s="13"/>
+      <c r="AR2" s="13"/>
+      <c r="AS2" s="13"/>
+      <c r="AT2" s="13"/>
+      <c r="AU2" s="13"/>
+      <c r="AV2" s="13"/>
+      <c r="AW2" s="13"/>
+      <c r="AX2" s="13"/>
+      <c r="AY2" s="13"/>
+      <c r="AZ2" s="13"/>
+      <c r="BA2" s="13"/>
+      <c r="BB2" s="13"/>
+      <c r="BC2" s="13"/>
+      <c r="BD2" s="13"/>
+      <c r="BE2" s="13"/>
+      <c r="BF2" s="13"/>
+      <c r="BG2" s="13"/>
+      <c r="BH2" s="13"/>
+      <c r="BI2" s="13"/>
+      <c r="BJ2" s="13"/>
+      <c r="BK2" s="13"/>
+      <c r="BL2" s="13"/>
+      <c r="BM2" s="13"/>
+      <c r="BN2" s="13"/>
+      <c r="BO2" s="13"/>
+      <c r="BP2" s="13"/>
+      <c r="BQ2" s="13"/>
+      <c r="BR2" s="13"/>
+      <c r="BS2" s="13"/>
+      <c r="BT2" s="13"/>
+      <c r="BU2" s="13"/>
+      <c r="BV2" s="13"/>
+      <c r="BW2" s="13"/>
+      <c r="BX2" s="13"/>
+      <c r="BY2" s="13"/>
+      <c r="BZ2" s="13"/>
+      <c r="CA2" s="13"/>
+      <c r="CB2" s="13"/>
+      <c r="CC2" s="13"/>
+      <c r="CD2" s="13"/>
+      <c r="CE2" s="13"/>
+      <c r="CF2" s="13"/>
+      <c r="CG2" s="13"/>
+      <c r="CH2" s="13"/>
+      <c r="CI2" s="13"/>
+      <c r="CJ2" s="13"/>
+      <c r="CK2" s="13"/>
+      <c r="CL2" s="13"/>
+      <c r="CM2" s="13"/>
+      <c r="CN2" s="13"/>
+      <c r="CO2" s="13"/>
+      <c r="CP2" s="13"/>
+      <c r="CQ2" s="13"/>
+      <c r="CR2" s="13"/>
+      <c r="CS2" s="13"/>
+      <c r="CT2" s="13"/>
+      <c r="CU2" s="13"/>
+      <c r="CV2" s="13"/>
+      <c r="CW2" s="13"/>
+      <c r="CX2" s="13"/>
+      <c r="CY2" s="13"/>
+      <c r="CZ2" s="13"/>
+      <c r="DA2" s="13"/>
+      <c r="DB2" s="13"/>
+      <c r="DC2" s="13"/>
+      <c r="DD2" s="13"/>
+      <c r="DE2" s="13"/>
+      <c r="DF2" s="13"/>
+      <c r="DG2" s="13"/>
+      <c r="DH2" s="13"/>
+      <c r="DI2" s="13"/>
+      <c r="DJ2" s="13"/>
+      <c r="DK2" s="13"/>
+      <c r="DL2" s="13"/>
+      <c r="DM2" s="13"/>
+      <c r="XFD2" s="0"/>
     </row>
-    <row r="3" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
-        <v>100000003372</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="8" t="s">
+    <row r="3" customFormat="false" ht="54.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>15</v>
       </c>
+      <c r="C3" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>17</v>
+      </c>
       <c r="E3" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="12" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
+        <v>18</v>
+      </c>
+      <c r="F3" s="12"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="1"/>
+      <c r="W3" s="1"/>
+      <c r="X3" s="1"/>
+      <c r="Y3" s="1"/>
+      <c r="Z3" s="1"/>
+      <c r="AA3" s="1"/>
+      <c r="AB3" s="1"/>
+      <c r="AC3" s="1"/>
+      <c r="AD3" s="1"/>
+      <c r="AE3" s="1"/>
+      <c r="AF3" s="1"/>
+      <c r="AG3" s="1"/>
+      <c r="AH3" s="1"/>
+      <c r="AI3" s="1"/>
+      <c r="AJ3" s="1"/>
+      <c r="AK3" s="1"/>
+      <c r="AL3" s="1"/>
+      <c r="AM3" s="1"/>
+      <c r="AN3" s="1"/>
+      <c r="AO3" s="1"/>
+      <c r="AP3" s="1"/>
+      <c r="AQ3" s="1"/>
+      <c r="AR3" s="1"/>
+      <c r="AS3" s="1"/>
+      <c r="AT3" s="1"/>
+      <c r="AU3" s="1"/>
+      <c r="AV3" s="1"/>
+      <c r="AW3" s="1"/>
+      <c r="AX3" s="1"/>
+      <c r="AY3" s="1"/>
+      <c r="AZ3" s="1"/>
+      <c r="BA3" s="1"/>
+      <c r="BB3" s="1"/>
+      <c r="BC3" s="1"/>
+      <c r="BD3" s="1"/>
+      <c r="BE3" s="1"/>
+      <c r="BF3" s="1"/>
+      <c r="BG3" s="1"/>
+      <c r="BH3" s="1"/>
+      <c r="BI3" s="1"/>
+      <c r="BJ3" s="1"/>
+      <c r="BK3" s="1"/>
+      <c r="BL3" s="1"/>
+      <c r="BM3" s="1"/>
+      <c r="BN3" s="1"/>
+      <c r="BO3" s="1"/>
+      <c r="BP3" s="1"/>
+      <c r="BQ3" s="1"/>
+      <c r="BR3" s="1"/>
+      <c r="BS3" s="1"/>
+      <c r="BT3" s="1"/>
+      <c r="BU3" s="1"/>
+      <c r="BV3" s="1"/>
+      <c r="BW3" s="1"/>
+      <c r="BX3" s="1"/>
+      <c r="BY3" s="1"/>
+      <c r="BZ3" s="1"/>
+      <c r="CA3" s="1"/>
+      <c r="CB3" s="1"/>
+      <c r="CC3" s="1"/>
+      <c r="CD3" s="1"/>
+      <c r="CE3" s="1"/>
+      <c r="CF3" s="1"/>
+      <c r="CG3" s="1"/>
+      <c r="CH3" s="1"/>
+      <c r="CI3" s="1"/>
+      <c r="CJ3" s="1"/>
+      <c r="CK3" s="1"/>
+      <c r="CL3" s="1"/>
+      <c r="CM3" s="1"/>
+      <c r="CN3" s="1"/>
+      <c r="CO3" s="1"/>
+      <c r="CP3" s="1"/>
+      <c r="CQ3" s="1"/>
+      <c r="CR3" s="1"/>
+      <c r="CS3" s="1"/>
+      <c r="CT3" s="1"/>
+      <c r="CU3" s="1"/>
+      <c r="CV3" s="1"/>
+      <c r="CW3" s="1"/>
+      <c r="CX3" s="1"/>
+      <c r="CY3" s="1"/>
+      <c r="CZ3" s="1"/>
+      <c r="DA3" s="1"/>
+      <c r="DB3" s="1"/>
+      <c r="DC3" s="1"/>
+      <c r="DD3" s="1"/>
+      <c r="DE3" s="1"/>
+      <c r="DF3" s="1"/>
+      <c r="DG3" s="1"/>
+      <c r="DH3" s="1"/>
+      <c r="DI3" s="1"/>
+      <c r="DJ3" s="1"/>
+      <c r="DK3" s="1"/>
+      <c r="DL3" s="1"/>
+      <c r="DM3" s="1"/>
+      <c r="XFD3" s="0"/>
     </row>
+    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="17"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="18"/>
+      <c r="R4" s="18"/>
+      <c r="S4" s="18"/>
+      <c r="T4" s="18"/>
+      <c r="U4" s="18"/>
+      <c r="V4" s="18"/>
+      <c r="W4" s="18"/>
+      <c r="X4" s="18"/>
+      <c r="Y4" s="18"/>
+      <c r="Z4" s="18"/>
+      <c r="AA4" s="18"/>
+      <c r="AB4" s="18"/>
+      <c r="AC4" s="18"/>
+      <c r="AD4" s="18"/>
+      <c r="AE4" s="18"/>
+      <c r="AF4" s="18"/>
+      <c r="AG4" s="18"/>
+      <c r="AH4" s="18"/>
+      <c r="AI4" s="18"/>
+      <c r="AJ4" s="18"/>
+      <c r="AK4" s="18"/>
+      <c r="AL4" s="18"/>
+      <c r="AM4" s="18"/>
+      <c r="AN4" s="18"/>
+      <c r="AO4" s="18"/>
+      <c r="AP4" s="18"/>
+      <c r="AQ4" s="18"/>
+      <c r="AR4" s="18"/>
+      <c r="AS4" s="18"/>
+      <c r="AT4" s="18"/>
+      <c r="AU4" s="18"/>
+      <c r="AV4" s="18"/>
+      <c r="AW4" s="18"/>
+      <c r="AX4" s="18"/>
+      <c r="AY4" s="18"/>
+      <c r="AZ4" s="18"/>
+      <c r="BA4" s="18"/>
+      <c r="BB4" s="18"/>
+      <c r="BC4" s="18"/>
+      <c r="BD4" s="18"/>
+      <c r="BE4" s="18"/>
+      <c r="BF4" s="18"/>
+      <c r="BG4" s="18"/>
+      <c r="BH4" s="18"/>
+      <c r="BI4" s="18"/>
+      <c r="BJ4" s="18"/>
+      <c r="BK4" s="18"/>
+      <c r="BL4" s="18"/>
+      <c r="BM4" s="18"/>
+      <c r="BN4" s="18"/>
+      <c r="BO4" s="18"/>
+      <c r="BP4" s="18"/>
+      <c r="BQ4" s="18"/>
+      <c r="BR4" s="18"/>
+      <c r="BS4" s="18"/>
+      <c r="BT4" s="18"/>
+      <c r="BU4" s="18"/>
+      <c r="BV4" s="18"/>
+      <c r="BW4" s="18"/>
+      <c r="BX4" s="18"/>
+      <c r="BY4" s="18"/>
+      <c r="BZ4" s="18"/>
+      <c r="CA4" s="18"/>
+      <c r="CB4" s="18"/>
+      <c r="CC4" s="18"/>
+      <c r="CD4" s="18"/>
+      <c r="CE4" s="18"/>
+      <c r="CF4" s="18"/>
+      <c r="CG4" s="18"/>
+      <c r="CH4" s="18"/>
+      <c r="CI4" s="18"/>
+      <c r="CJ4" s="18"/>
+      <c r="CK4" s="18"/>
+      <c r="CL4" s="18"/>
+      <c r="CM4" s="18"/>
+      <c r="CN4" s="18"/>
+      <c r="CO4" s="18"/>
+      <c r="CP4" s="18"/>
+      <c r="CQ4" s="18"/>
+      <c r="CR4" s="18"/>
+      <c r="CS4" s="18"/>
+      <c r="CT4" s="18"/>
+      <c r="CU4" s="18"/>
+      <c r="CV4" s="18"/>
+      <c r="CW4" s="18"/>
+      <c r="CX4" s="18"/>
+      <c r="CY4" s="18"/>
+      <c r="CZ4" s="18"/>
+      <c r="DA4" s="18"/>
+      <c r="DB4" s="18"/>
+      <c r="DC4" s="18"/>
+      <c r="DD4" s="18"/>
+      <c r="DE4" s="18"/>
+      <c r="DF4" s="18"/>
+      <c r="DG4" s="18"/>
+      <c r="DH4" s="18"/>
+      <c r="DI4" s="18"/>
+      <c r="DJ4" s="18"/>
+      <c r="DK4" s="18"/>
+      <c r="DL4" s="18"/>
+      <c r="DM4" s="18"/>
+      <c r="XFD4" s="0"/>
+    </row>
+    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>45510</v>
+      </c>
+      <c r="F5" s="12"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
+      <c r="Q5" s="13"/>
+      <c r="R5" s="13"/>
+      <c r="S5" s="13"/>
+      <c r="T5" s="13"/>
+      <c r="U5" s="13"/>
+      <c r="V5" s="13"/>
+      <c r="W5" s="13"/>
+      <c r="X5" s="13"/>
+      <c r="Y5" s="13"/>
+      <c r="Z5" s="13"/>
+      <c r="AA5" s="13"/>
+      <c r="AB5" s="13"/>
+      <c r="AC5" s="13"/>
+      <c r="AD5" s="13"/>
+      <c r="AE5" s="13"/>
+      <c r="AF5" s="13"/>
+      <c r="AG5" s="13"/>
+      <c r="AH5" s="13"/>
+      <c r="AI5" s="13"/>
+      <c r="AJ5" s="13"/>
+      <c r="AK5" s="13"/>
+      <c r="AL5" s="13"/>
+      <c r="AM5" s="13"/>
+      <c r="AN5" s="13"/>
+      <c r="AO5" s="13"/>
+      <c r="AP5" s="13"/>
+      <c r="AQ5" s="13"/>
+      <c r="AR5" s="13"/>
+      <c r="AS5" s="13"/>
+      <c r="AT5" s="13"/>
+      <c r="AU5" s="13"/>
+      <c r="AV5" s="13"/>
+      <c r="AW5" s="13"/>
+      <c r="AX5" s="13"/>
+      <c r="AY5" s="13"/>
+      <c r="AZ5" s="13"/>
+      <c r="BA5" s="13"/>
+      <c r="BB5" s="13"/>
+      <c r="BC5" s="13"/>
+      <c r="BD5" s="13"/>
+      <c r="BE5" s="13"/>
+      <c r="BF5" s="13"/>
+      <c r="BG5" s="13"/>
+      <c r="BH5" s="13"/>
+      <c r="BI5" s="13"/>
+      <c r="BJ5" s="13"/>
+      <c r="BK5" s="13"/>
+      <c r="BL5" s="13"/>
+      <c r="BM5" s="13"/>
+      <c r="BN5" s="13"/>
+      <c r="BO5" s="13"/>
+      <c r="BP5" s="13"/>
+      <c r="BQ5" s="13"/>
+      <c r="BR5" s="13"/>
+      <c r="BS5" s="13"/>
+      <c r="BT5" s="13"/>
+      <c r="BU5" s="13"/>
+      <c r="BV5" s="13"/>
+      <c r="BW5" s="13"/>
+      <c r="BX5" s="13"/>
+      <c r="BY5" s="13"/>
+      <c r="BZ5" s="13"/>
+      <c r="CA5" s="13"/>
+      <c r="CB5" s="13"/>
+      <c r="CC5" s="13"/>
+      <c r="CD5" s="13"/>
+      <c r="CE5" s="13"/>
+      <c r="CF5" s="13"/>
+      <c r="CG5" s="13"/>
+      <c r="CH5" s="13"/>
+      <c r="CI5" s="13"/>
+      <c r="CJ5" s="13"/>
+      <c r="CK5" s="13"/>
+      <c r="CL5" s="13"/>
+      <c r="CM5" s="13"/>
+      <c r="CN5" s="13"/>
+      <c r="CO5" s="13"/>
+      <c r="CP5" s="13"/>
+      <c r="CQ5" s="13"/>
+      <c r="CR5" s="13"/>
+      <c r="CS5" s="13"/>
+      <c r="CT5" s="13"/>
+      <c r="CU5" s="13"/>
+      <c r="CV5" s="13"/>
+      <c r="CW5" s="13"/>
+      <c r="CX5" s="13"/>
+      <c r="CY5" s="13"/>
+      <c r="CZ5" s="13"/>
+      <c r="DA5" s="13"/>
+      <c r="DB5" s="13"/>
+      <c r="DC5" s="13"/>
+      <c r="DD5" s="13"/>
+      <c r="DE5" s="13"/>
+      <c r="DF5" s="13"/>
+      <c r="DG5" s="13"/>
+      <c r="DH5" s="13"/>
+      <c r="DI5" s="13"/>
+      <c r="DJ5" s="13"/>
+      <c r="DK5" s="13"/>
+      <c r="DL5" s="13"/>
+      <c r="DM5" s="13"/>
+      <c r="XFD5" s="0"/>
+    </row>
+    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>46111</v>
+      </c>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="18"/>
+      <c r="T6" s="18"/>
+      <c r="U6" s="18"/>
+      <c r="V6" s="18"/>
+      <c r="W6" s="18"/>
+      <c r="X6" s="18"/>
+      <c r="Y6" s="18"/>
+      <c r="Z6" s="18"/>
+      <c r="AA6" s="18"/>
+      <c r="AB6" s="18"/>
+      <c r="AC6" s="18"/>
+      <c r="AD6" s="18"/>
+      <c r="AE6" s="18"/>
+      <c r="AF6" s="18"/>
+      <c r="AG6" s="18"/>
+      <c r="AH6" s="18"/>
+      <c r="AI6" s="18"/>
+      <c r="AJ6" s="18"/>
+      <c r="AK6" s="18"/>
+      <c r="AL6" s="18"/>
+      <c r="AM6" s="18"/>
+      <c r="AN6" s="18"/>
+      <c r="AO6" s="18"/>
+      <c r="AP6" s="18"/>
+      <c r="AQ6" s="18"/>
+      <c r="AR6" s="18"/>
+      <c r="AS6" s="18"/>
+      <c r="AT6" s="18"/>
+      <c r="AU6" s="18"/>
+      <c r="AV6" s="18"/>
+      <c r="AW6" s="18"/>
+      <c r="AX6" s="18"/>
+      <c r="AY6" s="18"/>
+      <c r="AZ6" s="18"/>
+      <c r="BA6" s="18"/>
+      <c r="BB6" s="18"/>
+      <c r="BC6" s="18"/>
+      <c r="BD6" s="18"/>
+      <c r="BE6" s="18"/>
+      <c r="BF6" s="18"/>
+      <c r="BG6" s="18"/>
+      <c r="BH6" s="18"/>
+      <c r="BI6" s="18"/>
+      <c r="BJ6" s="18"/>
+      <c r="BK6" s="18"/>
+      <c r="BL6" s="18"/>
+      <c r="BM6" s="18"/>
+      <c r="BN6" s="18"/>
+      <c r="BO6" s="18"/>
+      <c r="BP6" s="18"/>
+      <c r="BQ6" s="18"/>
+      <c r="BR6" s="18"/>
+      <c r="BS6" s="18"/>
+      <c r="BT6" s="18"/>
+      <c r="BU6" s="18"/>
+      <c r="BV6" s="18"/>
+      <c r="BW6" s="18"/>
+      <c r="BX6" s="18"/>
+      <c r="BY6" s="18"/>
+      <c r="BZ6" s="18"/>
+      <c r="CA6" s="18"/>
+      <c r="CB6" s="18"/>
+      <c r="CC6" s="18"/>
+      <c r="CD6" s="18"/>
+      <c r="CE6" s="18"/>
+      <c r="CF6" s="18"/>
+      <c r="CG6" s="18"/>
+      <c r="CH6" s="18"/>
+      <c r="CI6" s="18"/>
+      <c r="CJ6" s="18"/>
+      <c r="CK6" s="18"/>
+      <c r="CL6" s="18"/>
+      <c r="CM6" s="18"/>
+      <c r="CN6" s="18"/>
+      <c r="CO6" s="18"/>
+      <c r="CP6" s="18"/>
+      <c r="CQ6" s="18"/>
+      <c r="CR6" s="18"/>
+      <c r="CS6" s="18"/>
+      <c r="CT6" s="18"/>
+      <c r="CU6" s="18"/>
+      <c r="CV6" s="18"/>
+      <c r="CW6" s="18"/>
+      <c r="CX6" s="18"/>
+      <c r="CY6" s="18"/>
+      <c r="CZ6" s="18"/>
+      <c r="DA6" s="18"/>
+      <c r="DB6" s="18"/>
+      <c r="DC6" s="18"/>
+      <c r="DD6" s="18"/>
+      <c r="DE6" s="18"/>
+      <c r="DF6" s="18"/>
+      <c r="DG6" s="18"/>
+      <c r="DH6" s="18"/>
+      <c r="DI6" s="18"/>
+      <c r="DJ6" s="18"/>
+      <c r="DK6" s="18"/>
+      <c r="DL6" s="18"/>
+      <c r="DM6" s="18"/>
+      <c r="XFD6" s="0"/>
+    </row>
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>46111</v>
+      </c>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="13"/>
+      <c r="Q7" s="13"/>
+      <c r="R7" s="13"/>
+      <c r="S7" s="13"/>
+      <c r="T7" s="13"/>
+      <c r="U7" s="13"/>
+      <c r="V7" s="13"/>
+      <c r="W7" s="13"/>
+      <c r="X7" s="13"/>
+      <c r="Y7" s="13"/>
+      <c r="Z7" s="13"/>
+      <c r="AA7" s="13"/>
+      <c r="AB7" s="13"/>
+      <c r="AC7" s="13"/>
+      <c r="AD7" s="13"/>
+      <c r="AE7" s="13"/>
+      <c r="AF7" s="13"/>
+      <c r="AG7" s="13"/>
+      <c r="AH7" s="13"/>
+      <c r="AI7" s="13"/>
+      <c r="AJ7" s="13"/>
+      <c r="AK7" s="13"/>
+      <c r="AL7" s="13"/>
+      <c r="AM7" s="13"/>
+      <c r="AN7" s="13"/>
+      <c r="AO7" s="13"/>
+      <c r="AP7" s="13"/>
+      <c r="AQ7" s="13"/>
+      <c r="AR7" s="13"/>
+      <c r="AS7" s="13"/>
+      <c r="AT7" s="13"/>
+      <c r="AU7" s="13"/>
+      <c r="AV7" s="13"/>
+      <c r="AW7" s="13"/>
+      <c r="AX7" s="13"/>
+      <c r="AY7" s="13"/>
+      <c r="AZ7" s="13"/>
+      <c r="BA7" s="13"/>
+      <c r="BB7" s="13"/>
+      <c r="BC7" s="13"/>
+      <c r="BD7" s="13"/>
+      <c r="BE7" s="13"/>
+      <c r="BF7" s="13"/>
+      <c r="BG7" s="13"/>
+      <c r="BH7" s="13"/>
+      <c r="BI7" s="13"/>
+      <c r="BJ7" s="13"/>
+      <c r="BK7" s="13"/>
+      <c r="BL7" s="13"/>
+      <c r="BM7" s="13"/>
+      <c r="BN7" s="13"/>
+      <c r="BO7" s="13"/>
+      <c r="BP7" s="13"/>
+      <c r="BQ7" s="13"/>
+      <c r="BR7" s="13"/>
+      <c r="BS7" s="13"/>
+      <c r="BT7" s="13"/>
+      <c r="BU7" s="13"/>
+      <c r="BV7" s="13"/>
+      <c r="BW7" s="13"/>
+      <c r="BX7" s="13"/>
+      <c r="BY7" s="13"/>
+      <c r="BZ7" s="13"/>
+      <c r="CA7" s="13"/>
+      <c r="CB7" s="13"/>
+      <c r="CC7" s="13"/>
+      <c r="CD7" s="13"/>
+      <c r="CE7" s="13"/>
+      <c r="CF7" s="13"/>
+      <c r="CG7" s="13"/>
+      <c r="CH7" s="13"/>
+      <c r="CI7" s="13"/>
+      <c r="CJ7" s="13"/>
+      <c r="CK7" s="13"/>
+      <c r="CL7" s="13"/>
+      <c r="CM7" s="13"/>
+      <c r="CN7" s="13"/>
+      <c r="CO7" s="13"/>
+      <c r="CP7" s="13"/>
+      <c r="CQ7" s="13"/>
+      <c r="CR7" s="13"/>
+      <c r="CS7" s="13"/>
+      <c r="CT7" s="13"/>
+      <c r="CU7" s="13"/>
+      <c r="CV7" s="13"/>
+      <c r="CW7" s="13"/>
+      <c r="CX7" s="13"/>
+      <c r="CY7" s="13"/>
+      <c r="CZ7" s="13"/>
+      <c r="DA7" s="13"/>
+      <c r="DB7" s="13"/>
+      <c r="DC7" s="13"/>
+      <c r="DD7" s="13"/>
+      <c r="DE7" s="13"/>
+      <c r="DF7" s="13"/>
+      <c r="DG7" s="13"/>
+      <c r="DH7" s="13"/>
+      <c r="DI7" s="13"/>
+      <c r="DJ7" s="13"/>
+      <c r="DK7" s="13"/>
+      <c r="DL7" s="13"/>
+      <c r="DM7" s="13"/>
+      <c r="XFD7" s="0"/>
+    </row>
+    <row r="8" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="21"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="22"/>
+      <c r="R8" s="22"/>
+      <c r="S8" s="22"/>
+      <c r="T8" s="22"/>
+      <c r="U8" s="22"/>
+      <c r="V8" s="22"/>
+      <c r="W8" s="22"/>
+      <c r="X8" s="22"/>
+      <c r="Y8" s="22"/>
+      <c r="Z8" s="22"/>
+      <c r="AA8" s="22"/>
+      <c r="AB8" s="22"/>
+      <c r="AC8" s="22"/>
+      <c r="AD8" s="22"/>
+      <c r="AE8" s="22"/>
+      <c r="AF8" s="22"/>
+      <c r="AG8" s="22"/>
+      <c r="AH8" s="22"/>
+      <c r="AI8" s="22"/>
+      <c r="AJ8" s="22"/>
+      <c r="AK8" s="22"/>
+      <c r="AL8" s="22"/>
+      <c r="AM8" s="22"/>
+      <c r="AN8" s="22"/>
+      <c r="AO8" s="22"/>
+      <c r="AP8" s="22"/>
+      <c r="AQ8" s="22"/>
+      <c r="AR8" s="22"/>
+      <c r="AS8" s="22"/>
+      <c r="AT8" s="22"/>
+      <c r="AU8" s="22"/>
+      <c r="AV8" s="22"/>
+      <c r="AW8" s="22"/>
+      <c r="AX8" s="22"/>
+      <c r="AY8" s="22"/>
+      <c r="AZ8" s="22"/>
+      <c r="BA8" s="22"/>
+      <c r="BB8" s="22"/>
+      <c r="BC8" s="22"/>
+      <c r="BD8" s="22"/>
+      <c r="BE8" s="22"/>
+      <c r="BF8" s="22"/>
+      <c r="BG8" s="22"/>
+      <c r="BH8" s="22"/>
+      <c r="BI8" s="22"/>
+      <c r="BJ8" s="22"/>
+      <c r="BK8" s="22"/>
+      <c r="BL8" s="22"/>
+      <c r="BM8" s="22"/>
+      <c r="BN8" s="22"/>
+      <c r="BO8" s="22"/>
+      <c r="BP8" s="22"/>
+      <c r="BQ8" s="22"/>
+      <c r="BR8" s="22"/>
+      <c r="BS8" s="22"/>
+      <c r="BT8" s="22"/>
+      <c r="BU8" s="22"/>
+      <c r="BV8" s="22"/>
+      <c r="BW8" s="22"/>
+      <c r="BX8" s="22"/>
+      <c r="BY8" s="22"/>
+      <c r="BZ8" s="22"/>
+      <c r="CA8" s="22"/>
+      <c r="CB8" s="22"/>
+      <c r="CC8" s="22"/>
+      <c r="CD8" s="22"/>
+      <c r="CE8" s="22"/>
+      <c r="CF8" s="22"/>
+      <c r="CG8" s="22"/>
+      <c r="CH8" s="22"/>
+      <c r="CI8" s="22"/>
+      <c r="CJ8" s="22"/>
+      <c r="CK8" s="22"/>
+      <c r="CL8" s="22"/>
+      <c r="CM8" s="22"/>
+      <c r="CN8" s="22"/>
+      <c r="CO8" s="22"/>
+      <c r="CP8" s="22"/>
+      <c r="CQ8" s="22"/>
+      <c r="CR8" s="22"/>
+      <c r="CS8" s="22"/>
+      <c r="CT8" s="22"/>
+      <c r="CU8" s="22"/>
+      <c r="CV8" s="22"/>
+      <c r="CW8" s="22"/>
+      <c r="CX8" s="22"/>
+      <c r="CY8" s="22"/>
+      <c r="CZ8" s="22"/>
+      <c r="DA8" s="22"/>
+      <c r="DB8" s="22"/>
+      <c r="DC8" s="22"/>
+      <c r="DD8" s="22"/>
+      <c r="DE8" s="22"/>
+      <c r="DF8" s="22"/>
+      <c r="DG8" s="22"/>
+      <c r="DH8" s="22"/>
+      <c r="DI8" s="22"/>
+      <c r="DJ8" s="22"/>
+      <c r="DK8" s="22"/>
+      <c r="DL8" s="22"/>
+      <c r="DM8" s="22"/>
+      <c r="XFD8" s="0"/>
+    </row>
+    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
+      <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18"/>
+      <c r="R9" s="18"/>
+      <c r="S9" s="18"/>
+      <c r="T9" s="18"/>
+      <c r="U9" s="18"/>
+      <c r="V9" s="18"/>
+      <c r="W9" s="18"/>
+      <c r="X9" s="18"/>
+      <c r="Y9" s="18"/>
+      <c r="Z9" s="18"/>
+      <c r="AA9" s="18"/>
+      <c r="AB9" s="18"/>
+      <c r="AC9" s="18"/>
+      <c r="AD9" s="18"/>
+      <c r="AE9" s="18"/>
+      <c r="AF9" s="18"/>
+      <c r="AG9" s="18"/>
+      <c r="AH9" s="18"/>
+      <c r="AI9" s="18"/>
+      <c r="AJ9" s="18"/>
+      <c r="AK9" s="18"/>
+      <c r="AL9" s="18"/>
+      <c r="AM9" s="18"/>
+      <c r="AN9" s="18"/>
+      <c r="AO9" s="18"/>
+      <c r="AP9" s="18"/>
+      <c r="AQ9" s="18"/>
+      <c r="AR9" s="18"/>
+      <c r="AS9" s="18"/>
+      <c r="AT9" s="18"/>
+      <c r="AU9" s="18"/>
+      <c r="AV9" s="18"/>
+      <c r="AW9" s="18"/>
+      <c r="AX9" s="18"/>
+      <c r="AY9" s="18"/>
+      <c r="AZ9" s="18"/>
+      <c r="BA9" s="18"/>
+      <c r="BB9" s="18"/>
+      <c r="BC9" s="18"/>
+      <c r="BD9" s="18"/>
+      <c r="BE9" s="18"/>
+      <c r="BF9" s="18"/>
+      <c r="BG9" s="18"/>
+      <c r="BH9" s="18"/>
+      <c r="BI9" s="18"/>
+      <c r="BJ9" s="18"/>
+      <c r="BK9" s="18"/>
+      <c r="BL9" s="18"/>
+      <c r="BM9" s="18"/>
+      <c r="BN9" s="18"/>
+      <c r="BO9" s="18"/>
+      <c r="BP9" s="18"/>
+      <c r="BQ9" s="18"/>
+      <c r="BR9" s="18"/>
+      <c r="BS9" s="18"/>
+      <c r="BT9" s="18"/>
+      <c r="BU9" s="18"/>
+      <c r="BV9" s="18"/>
+      <c r="BW9" s="18"/>
+      <c r="BX9" s="18"/>
+      <c r="BY9" s="18"/>
+      <c r="BZ9" s="18"/>
+      <c r="CA9" s="18"/>
+      <c r="CB9" s="18"/>
+      <c r="CC9" s="18"/>
+      <c r="CD9" s="18"/>
+      <c r="CE9" s="18"/>
+      <c r="CF9" s="18"/>
+      <c r="CG9" s="18"/>
+      <c r="CH9" s="18"/>
+      <c r="CI9" s="18"/>
+      <c r="CJ9" s="18"/>
+      <c r="CK9" s="18"/>
+      <c r="CL9" s="18"/>
+      <c r="CM9" s="18"/>
+      <c r="CN9" s="18"/>
+      <c r="CO9" s="18"/>
+      <c r="CP9" s="18"/>
+      <c r="CQ9" s="18"/>
+      <c r="CR9" s="18"/>
+      <c r="CS9" s="18"/>
+      <c r="CT9" s="18"/>
+      <c r="CU9" s="18"/>
+      <c r="CV9" s="18"/>
+      <c r="CW9" s="18"/>
+      <c r="CX9" s="18"/>
+      <c r="CY9" s="18"/>
+      <c r="CZ9" s="18"/>
+      <c r="DA9" s="18"/>
+      <c r="DB9" s="18"/>
+      <c r="DC9" s="18"/>
+      <c r="DD9" s="18"/>
+      <c r="DE9" s="18"/>
+      <c r="DF9" s="18"/>
+      <c r="DG9" s="18"/>
+      <c r="DH9" s="18"/>
+      <c r="DI9" s="18"/>
+      <c r="DJ9" s="18"/>
+      <c r="DK9" s="18"/>
+      <c r="DL9" s="18"/>
+      <c r="DM9" s="18"/>
+      <c r="XFD9" s="0"/>
+    </row>
+    <row r="10" customFormat="false" ht="41.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="23"/>
+      <c r="F10" s="24" t="n">
+        <v>46122</v>
+      </c>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="13"/>
+      <c r="R10" s="13"/>
+      <c r="S10" s="13"/>
+      <c r="T10" s="13"/>
+      <c r="U10" s="13"/>
+      <c r="V10" s="13"/>
+      <c r="W10" s="13"/>
+      <c r="X10" s="13"/>
+      <c r="Y10" s="13"/>
+      <c r="Z10" s="13"/>
+      <c r="AA10" s="13"/>
+      <c r="AB10" s="13"/>
+      <c r="AC10" s="13"/>
+      <c r="AD10" s="13"/>
+      <c r="AE10" s="13"/>
+      <c r="AF10" s="13"/>
+      <c r="AG10" s="13"/>
+      <c r="AH10" s="13"/>
+      <c r="AI10" s="13"/>
+      <c r="AJ10" s="13"/>
+      <c r="AK10" s="13"/>
+      <c r="AL10" s="13"/>
+      <c r="AM10" s="13"/>
+      <c r="AN10" s="13"/>
+      <c r="AO10" s="13"/>
+      <c r="AP10" s="13"/>
+      <c r="AQ10" s="13"/>
+      <c r="AR10" s="13"/>
+      <c r="AS10" s="13"/>
+      <c r="AT10" s="13"/>
+      <c r="AU10" s="13"/>
+      <c r="AV10" s="13"/>
+      <c r="AW10" s="13"/>
+      <c r="AX10" s="13"/>
+      <c r="AY10" s="13"/>
+      <c r="AZ10" s="13"/>
+      <c r="BA10" s="13"/>
+      <c r="BB10" s="13"/>
+      <c r="BC10" s="13"/>
+      <c r="BD10" s="13"/>
+      <c r="BE10" s="13"/>
+      <c r="BF10" s="13"/>
+      <c r="BG10" s="13"/>
+      <c r="BH10" s="13"/>
+      <c r="BI10" s="13"/>
+      <c r="BJ10" s="13"/>
+      <c r="BK10" s="13"/>
+      <c r="BL10" s="13"/>
+      <c r="BM10" s="13"/>
+      <c r="BN10" s="13"/>
+      <c r="BO10" s="13"/>
+      <c r="BP10" s="13"/>
+      <c r="BQ10" s="13"/>
+      <c r="BR10" s="13"/>
+      <c r="BS10" s="13"/>
+      <c r="BT10" s="13"/>
+      <c r="BU10" s="13"/>
+      <c r="BV10" s="13"/>
+      <c r="BW10" s="13"/>
+      <c r="BX10" s="13"/>
+      <c r="BY10" s="13"/>
+      <c r="BZ10" s="13"/>
+      <c r="CA10" s="13"/>
+      <c r="CB10" s="13"/>
+      <c r="CC10" s="13"/>
+      <c r="CD10" s="13"/>
+      <c r="CE10" s="13"/>
+      <c r="CF10" s="13"/>
+      <c r="CG10" s="13"/>
+      <c r="CH10" s="13"/>
+      <c r="CI10" s="13"/>
+      <c r="CJ10" s="13"/>
+      <c r="CK10" s="13"/>
+      <c r="CL10" s="13"/>
+      <c r="CM10" s="13"/>
+      <c r="CN10" s="13"/>
+      <c r="CO10" s="13"/>
+      <c r="CP10" s="13"/>
+      <c r="CQ10" s="13"/>
+      <c r="CR10" s="13"/>
+      <c r="CS10" s="13"/>
+      <c r="CT10" s="13"/>
+      <c r="CU10" s="13"/>
+      <c r="CV10" s="13"/>
+      <c r="CW10" s="13"/>
+      <c r="CX10" s="13"/>
+      <c r="CY10" s="13"/>
+      <c r="CZ10" s="13"/>
+      <c r="DA10" s="13"/>
+      <c r="DB10" s="13"/>
+      <c r="DC10" s="13"/>
+      <c r="DD10" s="13"/>
+      <c r="DE10" s="13"/>
+      <c r="DF10" s="13"/>
+      <c r="DG10" s="13"/>
+      <c r="DH10" s="13"/>
+      <c r="DI10" s="13"/>
+      <c r="DJ10" s="13"/>
+      <c r="DK10" s="13"/>
+      <c r="DL10" s="13"/>
+      <c r="DM10" s="13"/>
+      <c r="XFD10" s="0"/>
+    </row>
+    <row r="11" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="21"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="28"/>
+      <c r="L11" s="28"/>
+      <c r="M11" s="28"/>
+      <c r="N11" s="28"/>
+      <c r="O11" s="28"/>
+      <c r="P11" s="28"/>
+      <c r="Q11" s="28"/>
+      <c r="R11" s="28"/>
+      <c r="S11" s="28"/>
+      <c r="T11" s="28"/>
+      <c r="U11" s="28"/>
+      <c r="V11" s="28"/>
+      <c r="W11" s="28"/>
+      <c r="X11" s="28"/>
+      <c r="Y11" s="28"/>
+      <c r="Z11" s="28"/>
+      <c r="AA11" s="28"/>
+      <c r="AB11" s="28"/>
+      <c r="AC11" s="28"/>
+      <c r="AD11" s="28"/>
+      <c r="AE11" s="28"/>
+      <c r="AF11" s="28"/>
+      <c r="AG11" s="28"/>
+      <c r="AH11" s="28"/>
+      <c r="AI11" s="28"/>
+      <c r="AJ11" s="28"/>
+      <c r="AK11" s="28"/>
+      <c r="AL11" s="28"/>
+      <c r="AM11" s="28"/>
+      <c r="AN11" s="28"/>
+      <c r="AO11" s="28"/>
+      <c r="AP11" s="28"/>
+      <c r="AQ11" s="28"/>
+      <c r="AR11" s="28"/>
+      <c r="AS11" s="28"/>
+      <c r="AT11" s="28"/>
+      <c r="AU11" s="28"/>
+      <c r="AV11" s="28"/>
+      <c r="AW11" s="28"/>
+      <c r="AX11" s="28"/>
+      <c r="AY11" s="28"/>
+      <c r="AZ11" s="28"/>
+      <c r="BA11" s="28"/>
+      <c r="BB11" s="28"/>
+      <c r="BC11" s="28"/>
+      <c r="BD11" s="28"/>
+      <c r="BE11" s="28"/>
+      <c r="BF11" s="28"/>
+      <c r="BG11" s="28"/>
+      <c r="BH11" s="28"/>
+      <c r="BI11" s="28"/>
+      <c r="BJ11" s="28"/>
+      <c r="BK11" s="28"/>
+      <c r="BL11" s="28"/>
+      <c r="BM11" s="28"/>
+      <c r="BN11" s="28"/>
+      <c r="BO11" s="28"/>
+      <c r="BP11" s="28"/>
+      <c r="BQ11" s="28"/>
+      <c r="BR11" s="28"/>
+      <c r="BS11" s="28"/>
+      <c r="BT11" s="28"/>
+      <c r="BU11" s="28"/>
+      <c r="BV11" s="28"/>
+      <c r="BW11" s="28"/>
+      <c r="BX11" s="28"/>
+      <c r="BY11" s="28"/>
+      <c r="BZ11" s="28"/>
+      <c r="CA11" s="28"/>
+      <c r="CB11" s="28"/>
+      <c r="CC11" s="28"/>
+      <c r="CD11" s="28"/>
+      <c r="CE11" s="28"/>
+      <c r="CF11" s="28"/>
+      <c r="CG11" s="28"/>
+      <c r="CH11" s="28"/>
+      <c r="CI11" s="28"/>
+      <c r="CJ11" s="28"/>
+      <c r="CK11" s="28"/>
+      <c r="CL11" s="28"/>
+      <c r="CM11" s="28"/>
+      <c r="CN11" s="28"/>
+      <c r="CO11" s="28"/>
+      <c r="CP11" s="28"/>
+      <c r="CQ11" s="28"/>
+      <c r="CR11" s="28"/>
+      <c r="CS11" s="28"/>
+      <c r="CT11" s="28"/>
+      <c r="CU11" s="28"/>
+      <c r="CV11" s="28"/>
+      <c r="CW11" s="28"/>
+      <c r="CX11" s="28"/>
+      <c r="CY11" s="28"/>
+      <c r="CZ11" s="28"/>
+      <c r="DA11" s="28"/>
+      <c r="DB11" s="28"/>
+      <c r="DC11" s="28"/>
+      <c r="DD11" s="28"/>
+      <c r="DE11" s="28"/>
+      <c r="DF11" s="28"/>
+      <c r="DG11" s="28"/>
+      <c r="DH11" s="28"/>
+      <c r="DI11" s="28"/>
+      <c r="DJ11" s="28"/>
+      <c r="DK11" s="28"/>
+      <c r="DL11" s="28"/>
+      <c r="DM11" s="28"/>
+      <c r="XFD11" s="0"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="29" t="n">
+        <v>57483</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="10"/>
+      <c r="E13" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F13" s="21"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="28"/>
+      <c r="K13" s="28"/>
+      <c r="L13" s="28"/>
+      <c r="M13" s="28"/>
+      <c r="N13" s="28"/>
+      <c r="O13" s="28"/>
+      <c r="P13" s="28"/>
+      <c r="Q13" s="28"/>
+      <c r="R13" s="28"/>
+      <c r="S13" s="28"/>
+      <c r="T13" s="28"/>
+      <c r="U13" s="28"/>
+      <c r="V13" s="28"/>
+      <c r="W13" s="28"/>
+      <c r="X13" s="28"/>
+      <c r="Y13" s="28"/>
+      <c r="Z13" s="28"/>
+      <c r="AA13" s="28"/>
+      <c r="AB13" s="28"/>
+      <c r="AC13" s="28"/>
+      <c r="AD13" s="28"/>
+      <c r="AE13" s="28"/>
+      <c r="AF13" s="28"/>
+      <c r="AG13" s="28"/>
+      <c r="AH13" s="28"/>
+      <c r="AI13" s="28"/>
+      <c r="AJ13" s="28"/>
+      <c r="AK13" s="28"/>
+      <c r="AL13" s="28"/>
+      <c r="AM13" s="28"/>
+      <c r="AN13" s="28"/>
+      <c r="AO13" s="28"/>
+      <c r="AP13" s="28"/>
+      <c r="AQ13" s="28"/>
+      <c r="AR13" s="28"/>
+      <c r="AS13" s="28"/>
+      <c r="AT13" s="28"/>
+      <c r="AU13" s="28"/>
+      <c r="AV13" s="28"/>
+      <c r="AW13" s="28"/>
+      <c r="AX13" s="28"/>
+      <c r="AY13" s="28"/>
+      <c r="AZ13" s="28"/>
+      <c r="BA13" s="28"/>
+      <c r="BB13" s="28"/>
+      <c r="BC13" s="28"/>
+      <c r="BD13" s="28"/>
+      <c r="BE13" s="28"/>
+      <c r="BF13" s="28"/>
+      <c r="BG13" s="28"/>
+      <c r="BH13" s="28"/>
+      <c r="BI13" s="28"/>
+      <c r="BJ13" s="28"/>
+      <c r="BK13" s="28"/>
+      <c r="BL13" s="28"/>
+      <c r="BM13" s="28"/>
+      <c r="BN13" s="28"/>
+      <c r="BO13" s="28"/>
+      <c r="BP13" s="28"/>
+      <c r="BQ13" s="28"/>
+      <c r="BR13" s="28"/>
+      <c r="BS13" s="28"/>
+      <c r="BT13" s="28"/>
+      <c r="BU13" s="28"/>
+      <c r="BV13" s="28"/>
+      <c r="BW13" s="28"/>
+      <c r="BX13" s="28"/>
+      <c r="BY13" s="28"/>
+      <c r="BZ13" s="28"/>
+      <c r="CA13" s="28"/>
+      <c r="CB13" s="28"/>
+      <c r="CC13" s="28"/>
+      <c r="CD13" s="28"/>
+      <c r="CE13" s="28"/>
+      <c r="CF13" s="28"/>
+      <c r="CG13" s="28"/>
+      <c r="CH13" s="28"/>
+      <c r="CI13" s="28"/>
+      <c r="CJ13" s="28"/>
+      <c r="CK13" s="28"/>
+      <c r="CL13" s="28"/>
+      <c r="CM13" s="28"/>
+      <c r="CN13" s="28"/>
+      <c r="CO13" s="28"/>
+      <c r="CP13" s="28"/>
+      <c r="CQ13" s="28"/>
+      <c r="CR13" s="28"/>
+      <c r="CS13" s="28"/>
+      <c r="CT13" s="28"/>
+      <c r="CU13" s="28"/>
+      <c r="CV13" s="28"/>
+      <c r="CW13" s="28"/>
+      <c r="CX13" s="28"/>
+      <c r="CY13" s="28"/>
+      <c r="CZ13" s="28"/>
+      <c r="DA13" s="28"/>
+      <c r="DB13" s="28"/>
+      <c r="DC13" s="28"/>
+      <c r="DD13" s="28"/>
+      <c r="DE13" s="28"/>
+      <c r="DF13" s="28"/>
+      <c r="DG13" s="28"/>
+      <c r="DH13" s="28"/>
+      <c r="DI13" s="28"/>
+      <c r="DJ13" s="28"/>
+      <c r="DK13" s="28"/>
+      <c r="DL13" s="28"/>
+      <c r="DM13" s="28"/>
+      <c r="XFD13" s="0"/>
+    </row>
+    <row r="1048331" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048332" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048333" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048334" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048335" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048336" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048337" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048338" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048339" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048340" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048341" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048342" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048343" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048344" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048345" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048346" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048347" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048348" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048349" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048350" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048352" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048353" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048354" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048356" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048357" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048358" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048359" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048360" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048361" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048362" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048363" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048364" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048365" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048366" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048367" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048368" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048369" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048370" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048371" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048372" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048373" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048374" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048375" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048376" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048377" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048379" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048380" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048381" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048382" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048383" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048384" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048385" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048386" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048387" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048389" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048390" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048391" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048392" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048394" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048395" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048396" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048397" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048398" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048399" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048400" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048401" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048402" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048403" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048404" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048405" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048406" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048407" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048408" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048409" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048410" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048411" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048412" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048413" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048414" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048415" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048418" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -886,6 +2704,38 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
+  <conditionalFormatting sqref="B11 B13">
+    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="0">
+      <formula>NOT(ISERROR(SEARCH("workstation",B11)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10">
+    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="1">
+      <formula>NOT(ISERROR(SEARCH("workstation",B10)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4">
+    <cfRule type="containsText" priority="4" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="2">
+      <formula>NOT(ISERROR(SEARCH("workstation",B4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="5" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="3">
+      <formula>NOT(ISERROR(SEARCH("workstation",B4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="6" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="4">
+      <formula>NOT(ISERROR(SEARCH("workstation",B4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="7" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="5">
+      <formula>NOT(ISERROR(SEARCH("workstation",B4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="8" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="6">
+      <formula>NOT(ISERROR(SEARCH("workstation",B4)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2">
+    <cfRule type="containsText" priority="9" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="workstation" dxfId="7">
+      <formula>NOT(ISERROR(SEARCH("workstation",B2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>